<commit_message>
Third batch of manually scraped adopted plans
</commit_message>
<xml_diff>
--- a/data/manually_scraped_adopted_plans.xlsx
+++ b/data/manually_scraped_adopted_plans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sianteesdale/Documents/GitHub/local-plan-extractor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4999ADE-3B9E-6747-B7F8-309A1BD086C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5BE992-0580-C548-BB29-47A7E5E1E80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="645">
   <si>
     <t>organisation</t>
   </si>
@@ -1854,9 +1854,6 @@
     <t>https://www.centralbedfordshire.gov.uk/info/153/central_bedfordshire_local_plan_2015_to_2035/1034/adopted_local_plan</t>
   </si>
   <si>
-    <t>https://centralbedfordshirecouncil.sharepoint.com/sites/Communications/Website and intranet/Forms/AllItems.aspx?id=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2FCentral%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2Epdf&amp;parent=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035&amp;p=true&amp;ga=1</t>
-  </si>
-  <si>
     <t>https://www.charnwood.gov.uk/pages/local_plan</t>
   </si>
   <si>
@@ -1875,9 +1872,6 @@
     <t>https://www.cheshirewestandchester.gov.uk/your-council/policies-and-performance/council-plans-policies-and-strategies/planning-policy/local-plan/local-plan-part-one</t>
   </si>
   <si>
-    <t>https://planningpolicy.cheshirewestandchester.gov.uk/sites/planningpolicy-cheshirewestandchester/files/2025-11/Local Plan %28Part One%29 Strategic Policies.pdf</t>
-  </si>
-  <si>
     <t>https://www.dacorum.gov.uk/docs/default-source/strategic-planning/adopted-core-strategy-2013.pdf?sfvrsn=80753a9e_2</t>
   </si>
   <si>
@@ -1978,6 +1972,12 @@
   </si>
   <si>
     <t>https://go.walsall.gov.uk/sites/default/files/2022-09/Black%20Country%20Core%20Strategy.pdf</t>
+  </si>
+  <si>
+    <t>https://centralbedfordshirecouncil.sharepoint.com/sites/Communications/Website%20and%20intranet/Forms/AllItems.aspx?id=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2FCentral%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2Epdf&amp;parent=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035&amp;p=true&amp;ga=1</t>
+  </si>
+  <si>
+    <t>https://planningpolicy.cheshirewestandchester.gov.uk/sites/planningpolicy-cheshirewestandchester/files/2025-11/Local%20Plan%20%28Part%20One%29%20Strategic%20Policies.pdf</t>
   </si>
 </sst>
 </file>
@@ -2426,7 +2426,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:O135"/>
+  <dimension ref="A1:Q135"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22.33203125" customWidth="1"/>
@@ -2582,7 +2582,7 @@
         <v>579</v>
       </c>
       <c r="E5" s="40" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F5" s="2">
         <v>2023</v>
@@ -2811,7 +2811,7 @@
         <v>590</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="F12" s="2">
         <v>2017</v>
@@ -2942,7 +2942,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="16">
+    <row r="17" spans="1:17" ht="16">
       <c r="A17" s="15" t="s">
         <v>53</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="16">
+    <row r="18" spans="1:17" ht="16">
       <c r="A18" s="15" t="s">
         <v>53</v>
       </c>
@@ -3000,7 +3000,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="16">
+    <row r="19" spans="1:17" ht="16">
       <c r="A19" s="15" t="s">
         <v>53</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="16">
+    <row r="20" spans="1:17" ht="16">
       <c r="A20" s="1" t="s">
         <v>60</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="16">
+    <row r="21" spans="1:17" ht="16">
       <c r="A21" s="1" t="s">
         <v>63</v>
       </c>
@@ -3068,11 +3068,11 @@
       <c r="C21" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="9" t="s">
+      <c r="D21" s="40" t="s">
         <v>602</v>
       </c>
-      <c r="E21" s="9" t="s">
-        <v>603</v>
+      <c r="E21" s="40" t="s">
+        <v>643</v>
       </c>
       <c r="F21" s="2">
         <v>2015</v>
@@ -3087,7 +3087,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="16">
+    <row r="22" spans="1:17" ht="16">
       <c r="A22" s="21" t="s">
         <v>66</v>
       </c>
@@ -3098,10 +3098,10 @@
         <v>27</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="E22" s="40" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F22" s="22">
         <v>2011</v>
@@ -3116,7 +3116,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="16">
+    <row r="23" spans="1:17" ht="16">
       <c r="A23" s="1" t="s">
         <v>69</v>
       </c>
@@ -3127,10 +3127,10 @@
         <v>27</v>
       </c>
       <c r="D23" s="9" t="s">
+        <v>604</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>605</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>606</v>
       </c>
       <c r="F23" s="2">
         <v>2010</v>
@@ -3145,7 +3145,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="16">
+    <row r="24" spans="1:17" ht="16">
       <c r="A24" s="1" t="s">
         <v>72</v>
       </c>
@@ -3156,10 +3156,10 @@
         <v>27</v>
       </c>
       <c r="D24" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="E24" s="9" t="s">
         <v>607</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>608</v>
       </c>
       <c r="F24" s="2">
         <v>2018</v>
@@ -3174,7 +3174,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="16">
+    <row r="25" spans="1:17" ht="16">
       <c r="A25" s="1" t="s">
         <v>75</v>
       </c>
@@ -3185,10 +3185,10 @@
         <v>27</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>609</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>610</v>
+        <v>608</v>
+      </c>
+      <c r="E25" s="40" t="s">
+        <v>644</v>
       </c>
       <c r="F25" s="2">
         <v>2015</v>
@@ -3203,7 +3203,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="16">
+    <row r="26" spans="1:17" ht="16">
       <c r="A26" s="1" t="s">
         <v>78</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="16">
+    <row r="27" spans="1:17" ht="16">
       <c r="A27" s="1" t="s">
         <v>84</v>
       </c>
@@ -3258,7 +3258,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="16">
+    <row r="28" spans="1:17" ht="16">
       <c r="A28" s="1" t="s">
         <v>88</v>
       </c>
@@ -3284,7 +3284,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="16">
+    <row r="29" spans="1:17" ht="16">
       <c r="A29" s="1" t="s">
         <v>92</v>
       </c>
@@ -3298,7 +3298,7 @@
         <v>94</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="F29" s="2">
         <v>2006</v>
@@ -3313,7 +3313,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="16">
+    <row r="30" spans="1:17" ht="16">
       <c r="A30" s="1" t="s">
         <v>96</v>
       </c>
@@ -3338,8 +3338,11 @@
       <c r="I30" s="6" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" ht="16">
+      <c r="Q30" s="46" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="16">
       <c r="A31" s="1" t="s">
         <v>100</v>
       </c>
@@ -3365,7 +3368,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="16">
+    <row r="32" spans="1:17" ht="16">
       <c r="A32" s="1" t="s">
         <v>104</v>
       </c>
@@ -3576,7 +3579,7 @@
         <v>27</v>
       </c>
       <c r="D39" s="42" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="E39" s="44" t="s">
         <v>126</v>
@@ -3793,10 +3796,10 @@
         <v>27</v>
       </c>
       <c r="D47" s="42" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F47" s="19">
         <v>2011</v>
@@ -3964,7 +3967,7 @@
         <v>179</v>
       </c>
       <c r="E53" s="40" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="F53" s="19">
         <v>2011</v>
@@ -3990,7 +3993,7 @@
         <v>27</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="E54" s="9" t="s">
         <v>183</v>
@@ -4395,10 +4398,10 @@
         <v>27</v>
       </c>
       <c r="D69" s="42" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E69" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="F69" s="19">
         <v>2014</v>
@@ -4424,10 +4427,10 @@
         <v>27</v>
       </c>
       <c r="D70" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="F70" s="19">
         <v>2023</v>
@@ -4505,10 +4508,10 @@
         <v>27</v>
       </c>
       <c r="D73" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E73" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F73" s="19">
         <v>2022</v>
@@ -4670,10 +4673,10 @@
         <v>27</v>
       </c>
       <c r="D79" s="42" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E79" s="47" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F79" s="19">
         <v>2011</v>
@@ -4699,10 +4702,10 @@
         <v>27</v>
       </c>
       <c r="D80" s="42" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="E80" s="47" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="F80" s="19">
         <v>2011</v>
@@ -4728,10 +4731,10 @@
         <v>27</v>
       </c>
       <c r="D81" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E81" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F81" s="19">
         <v>2022</v>
@@ -4809,10 +4812,10 @@
         <v>27</v>
       </c>
       <c r="D84" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E84" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F84" s="19">
         <v>2022</v>
@@ -4945,10 +4948,10 @@
         <v>27</v>
       </c>
       <c r="D89" s="42" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="E89" s="42" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="F89" s="19">
         <v>1994</v>
@@ -4974,10 +4977,10 @@
         <v>27</v>
       </c>
       <c r="D90" s="42" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="E90" s="42" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F90" s="19">
         <v>2011</v>
@@ -5185,10 +5188,10 @@
         <v>27</v>
       </c>
       <c r="D98" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E98" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F98" s="19">
         <v>2022</v>
@@ -5544,10 +5547,10 @@
         <v>27</v>
       </c>
       <c r="D111" s="42" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E111" s="42" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="F111" s="19">
         <v>2011</v>
@@ -5599,10 +5602,10 @@
         <v>27</v>
       </c>
       <c r="D113" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E113" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="F113" s="19">
         <v>2022</v>
@@ -5732,10 +5735,10 @@
         <v>27</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="E118" s="40" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="F118" s="19">
         <v>2011</v>
@@ -5761,10 +5764,10 @@
         <v>27</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="E119" s="40" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="F119" s="19">
         <v>2011</v>
@@ -6402,6 +6405,9 @@
     <hyperlink ref="E80" r:id="rId188" xr:uid="{0D57FF1B-9E12-8C47-A129-002F2009368C}"/>
     <hyperlink ref="E118" r:id="rId189" xr:uid="{EF87D15A-AB58-8D42-9CEA-BC13F4F645F7}"/>
     <hyperlink ref="E119" r:id="rId190" xr:uid="{851D742F-ABFD-344E-BD1E-FA41E5693714}"/>
+    <hyperlink ref="E21" r:id="rId191" display="https://centralbedfordshirecouncil.sharepoint.com/sites/Communications/Website and intranet/Forms/AllItems.aspx?id=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2FCentral%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2Epdf&amp;parent=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035&amp;p=true&amp;ga=1" xr:uid="{0A21C8F8-F7E2-ED4D-B000-E3B6AB33E60B}"/>
+    <hyperlink ref="D21" r:id="rId192" xr:uid="{F1D92A59-16C4-1E43-9906-76DB10045477}"/>
+    <hyperlink ref="E25" r:id="rId193" xr:uid="{B606F106-13F9-3143-9FAD-49CDAA46AED7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -6470,31 +6476,31 @@
         <v>7</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="6" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B9" s="46" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="6" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fourth batch of manually scraped adopted plans
</commit_message>
<xml_diff>
--- a/data/manually_scraped_adopted_plans.xlsx
+++ b/data/manually_scraped_adopted_plans.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sianteesdale/Documents/GitHub/local-plan-extractor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD5BE992-0580-C548-BB29-47A7E5E1E80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB11815-EDE9-2D42-A568-4C01F0A4E9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35800" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="manual-search" sheetId="1" r:id="rId1"/>
@@ -585,18 +585,6 @@
     <t>Gloucester City Council</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="10"/>
-        <color rgb="FF1155CC"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>gloucester.gov.uk/media/hgun5cpe/gloucester-city-plan-high-res.pdf</t>
-    </r>
-  </si>
-  <si>
     <t>Gloucester has a Joint Core Strategy with Cheltenham and Tewkesbury. It also has a Gloucester City Local Plan 2011 - 2031 adopted 2023.</t>
   </si>
   <si>
@@ -726,9 +714,6 @@
     <t>https://www.hounslow.gov.uk/local-plan/local-plan-1</t>
   </si>
   <si>
-    <t>https://lbhounslow.sharepoint.com/sites/InternetLinks/pp/Shared%20Documents/Forms/AllItems.aspx?id=%2Fsites%2FInternetLinks%2Fpp%2FShared%20Documents%2FPlanning%20and%20Building%20%28WEBPAGES%29%2FPlanning%20Policy%2FLocal%20Plan%2FLocal%20Plan%20%282015%29%2FHounslow%20Local%20Plan%20Part%201%20Direct%2Epdf&amp;parent=%2Fsites%2FInternetLinks%2Fpp%2FShared%20Documents%2FPlanning%20and%20Building%20%28WEBPAGES%29%2FPlanning%20Policy%2FLocal%20Plan%2FLocal%20Plan%20%282015%29&amp;p=true&amp;ga=1</t>
-  </si>
-  <si>
     <t>Sharepoint Doc - may need to manually download it</t>
   </si>
   <si>
@@ -1978,6 +1963,12 @@
   </si>
   <si>
     <t>https://planningpolicy.cheshirewestandchester.gov.uk/sites/planningpolicy-cheshirewestandchester/files/2025-11/Local%20Plan%20%28Part%20One%29%20Strategic%20Policies.pdf</t>
+  </si>
+  <si>
+    <t>https://gloucester.gov.uk/media/hgun5cpe/gloucester-city-plan-high-res.pdf</t>
+  </si>
+  <si>
+    <t>https://lbhounslow.sharepoint.com/:b:/s/InternetLinks/pp/EcHMd2lpx5xFlwDbyfEsUrcBvxzfTSoTrW3yOphnXdPQzg?e=fsgeqV</t>
   </si>
 </sst>
 </file>
@@ -2457,10 +2448,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>7</v>
@@ -2513,10 +2504,10 @@
         <v>18</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="F3" s="2">
         <v>2022</v>
@@ -2546,10 +2537,10 @@
         <v>18</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="F4" s="2">
         <v>2023</v>
@@ -2579,10 +2570,10 @@
         <v>27</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E5" s="40" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="F5" s="2">
         <v>2023</v>
@@ -2612,10 +2603,10 @@
         <v>27</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E6" s="40" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="F6" s="2">
         <v>2020</v>
@@ -2678,10 +2669,10 @@
         <v>27</v>
       </c>
       <c r="D8" s="41" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E8" s="41" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="F8" s="16">
         <v>2006</v>
@@ -2711,10 +2702,10 @@
         <v>27</v>
       </c>
       <c r="D9" s="41" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E9" s="41" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="F9" s="16">
         <v>2014</v>
@@ -2746,10 +2737,10 @@
         <v>27</v>
       </c>
       <c r="D10" s="41" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E10" s="41" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="F10" s="16">
         <v>2018</v>
@@ -2779,10 +2770,10 @@
         <v>27</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="E11" s="42" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="F11" s="19">
         <v>2022</v>
@@ -2808,10 +2799,10 @@
         <v>27</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="F12" s="2">
         <v>2017</v>
@@ -2837,10 +2828,10 @@
         <v>27</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="F13" s="2">
         <v>2011</v>
@@ -2866,10 +2857,10 @@
         <v>27</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="F14" s="2">
         <v>2011</v>
@@ -2924,10 +2915,10 @@
         <v>27</v>
       </c>
       <c r="D16" s="41" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E16" s="41" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="F16" s="16">
         <v>2013</v>
@@ -2953,10 +2944,10 @@
         <v>27</v>
       </c>
       <c r="D17" s="41" t="s">
+        <v>593</v>
+      </c>
+      <c r="E17" s="41" t="s">
         <v>595</v>
-      </c>
-      <c r="E17" s="41" t="s">
-        <v>597</v>
       </c>
       <c r="F17" s="16">
         <v>1997</v>
@@ -2982,10 +2973,10 @@
         <v>27</v>
       </c>
       <c r="D18" s="41" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E18" s="41" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="F18" s="16">
         <v>1999</v>
@@ -3011,10 +3002,10 @@
         <v>27</v>
       </c>
       <c r="D19" s="41" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="F19" s="16">
         <v>2019</v>
@@ -3040,10 +3031,10 @@
         <v>27</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="F20" s="2">
         <v>2012</v>
@@ -3069,10 +3060,10 @@
         <v>27</v>
       </c>
       <c r="D21" s="40" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="E21" s="40" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="F21" s="2">
         <v>2015</v>
@@ -3098,10 +3089,10 @@
         <v>27</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="E22" s="40" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F22" s="22">
         <v>2011</v>
@@ -3127,10 +3118,10 @@
         <v>27</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F23" s="2">
         <v>2010</v>
@@ -3156,10 +3147,10 @@
         <v>27</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="F24" s="2">
         <v>2018</v>
@@ -3185,10 +3176,10 @@
         <v>27</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="F25" s="2">
         <v>2015</v>
@@ -3298,7 +3289,7 @@
         <v>94</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="F29" s="2">
         <v>2006</v>
@@ -3339,7 +3330,7 @@
         <v>83</v>
       </c>
       <c r="Q30" s="46" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="16">
@@ -3579,7 +3570,7 @@
         <v>27</v>
       </c>
       <c r="D39" s="42" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="E39" s="44" t="s">
         <v>126</v>
@@ -3796,10 +3787,10 @@
         <v>27</v>
       </c>
       <c r="D47" s="42" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="F47" s="19">
         <v>2011</v>
@@ -3967,7 +3958,7 @@
         <v>179</v>
       </c>
       <c r="E53" s="40" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="F53" s="19">
         <v>2011</v>
@@ -3993,10 +3984,10 @@
         <v>27</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>612</v>
-      </c>
-      <c r="E54" s="9" t="s">
-        <v>183</v>
+        <v>610</v>
+      </c>
+      <c r="E54" s="40" t="s">
+        <v>643</v>
       </c>
       <c r="F54" s="19">
         <v>2011</v>
@@ -4005,7 +3996,7 @@
         <v>2031</v>
       </c>
       <c r="H54" s="18" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I54" s="6" t="s">
         <v>13</v>
@@ -4013,19 +4004,19 @@
     </row>
     <row r="55" spans="1:9" ht="16">
       <c r="A55" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="C55" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D55" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="C55" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D55" s="9" t="s">
+      <c r="E55" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="E55" s="9" t="s">
-        <v>188</v>
       </c>
       <c r="F55" s="2">
         <v>2011</v>
@@ -4039,19 +4030,19 @@
     </row>
     <row r="56" spans="1:9" ht="16">
       <c r="A56" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="C56" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D56" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C56" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D56" s="9" t="s">
+      <c r="E56" s="24" t="s">
         <v>191</v>
-      </c>
-      <c r="E56" s="24" t="s">
-        <v>192</v>
       </c>
       <c r="F56" s="2">
         <v>2015</v>
@@ -4065,19 +4056,19 @@
     </row>
     <row r="57" spans="1:9" ht="16">
       <c r="A57" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="C57" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D57" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="C57" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D57" s="9" t="s">
+      <c r="E57" s="9" t="s">
         <v>195</v>
-      </c>
-      <c r="E57" s="9" t="s">
-        <v>196</v>
       </c>
       <c r="F57" s="2">
         <v>2013</v>
@@ -4086,7 +4077,7 @@
         <v>2030</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="I57" s="6" t="s">
         <v>83</v>
@@ -4094,19 +4085,19 @@
     </row>
     <row r="58" spans="1:9" ht="16">
       <c r="A58" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="C58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D58" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D58" s="9" t="s">
+      <c r="E58" s="9" t="s">
         <v>200</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>201</v>
       </c>
       <c r="F58" s="2">
         <v>2014</v>
@@ -4115,7 +4106,7 @@
         <v>2037</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I58" s="6" t="s">
         <v>83</v>
@@ -4123,19 +4114,19 @@
     </row>
     <row r="59" spans="1:9" ht="16">
       <c r="A59" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="C59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D59" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D59" s="9" t="s">
+      <c r="E59" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="E59" s="9" t="s">
-        <v>206</v>
       </c>
       <c r="F59" s="2">
         <v>2011</v>
@@ -4149,19 +4140,19 @@
     </row>
     <row r="60" spans="1:9" ht="16">
       <c r="A60" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="C60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D60" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="C60" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D60" s="9" t="s">
+      <c r="E60" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="E60" s="9" t="s">
-        <v>210</v>
       </c>
       <c r="F60" s="2">
         <v>2016</v>
@@ -4175,19 +4166,19 @@
     </row>
     <row r="61" spans="1:9" ht="16">
       <c r="A61" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="C61" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D61" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D61" s="9" t="s">
+      <c r="E61" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="E61" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="F61" s="2">
         <v>2018</v>
@@ -4196,7 +4187,7 @@
         <v>2033</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I61" s="6" t="s">
         <v>83</v>
@@ -4204,19 +4195,19 @@
     </row>
     <row r="62" spans="1:9" ht="16">
       <c r="A62" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="C62" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D62" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="C62" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D62" s="9" t="s">
+      <c r="E62" s="9" t="s">
         <v>218</v>
-      </c>
-      <c r="E62" s="9" t="s">
-        <v>219</v>
       </c>
       <c r="F62" s="2">
         <v>2011</v>
@@ -4230,19 +4221,19 @@
     </row>
     <row r="63" spans="1:9" ht="16">
       <c r="A63" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="C63" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D63" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="C63" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D63" s="9" t="s">
+      <c r="E63" s="9" t="s">
         <v>222</v>
-      </c>
-      <c r="E63" s="9" t="s">
-        <v>223</v>
       </c>
       <c r="F63" s="2">
         <v>2011</v>
@@ -4256,19 +4247,19 @@
     </row>
     <row r="64" spans="1:9" ht="16">
       <c r="A64" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="C64" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D64" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="E64" s="9" t="s">
-        <v>227</v>
+      <c r="E64" s="40" t="s">
+        <v>644</v>
       </c>
       <c r="F64" s="2">
         <v>2015</v>
@@ -4277,7 +4268,7 @@
         <v>2030</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="I64" s="6" t="s">
         <v>83</v>
@@ -4285,19 +4276,19 @@
     </row>
     <row r="65" spans="1:9" ht="16">
       <c r="A65" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D65" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="E65" s="9" t="s">
         <v>230</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="E65" s="9" t="s">
-        <v>232</v>
       </c>
       <c r="F65" s="2">
         <v>2011</v>
@@ -4311,19 +4302,19 @@
     </row>
     <row r="66" spans="1:9" ht="16">
       <c r="A66" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D66" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="E66" s="24" t="s">
         <v>234</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D66" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="E66" s="24" t="s">
-        <v>236</v>
       </c>
       <c r="F66" s="2">
         <v>2016</v>
@@ -4337,19 +4328,19 @@
     </row>
     <row r="67" spans="1:9" ht="16">
       <c r="A67" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D67" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="E67" s="45" t="s">
         <v>238</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D67" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="E67" s="45" t="s">
-        <v>240</v>
       </c>
       <c r="F67" s="2">
         <v>2011</v>
@@ -4363,19 +4354,19 @@
     </row>
     <row r="68" spans="1:9" ht="16">
       <c r="A68" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D68" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="E68" s="24" t="s">
         <v>242</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D68" s="9" t="s">
-        <v>243</v>
-      </c>
-      <c r="E68" s="24" t="s">
-        <v>244</v>
       </c>
       <c r="F68" s="2">
         <v>2011</v>
@@ -4389,19 +4380,19 @@
     </row>
     <row r="69" spans="1:9" ht="16">
       <c r="A69" s="17" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C69" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D69" s="42" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="E69" s="42" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="F69" s="19">
         <v>2014</v>
@@ -4410,7 +4401,7 @@
         <v>2026</v>
       </c>
       <c r="H69" s="18" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I69" s="6" t="s">
         <v>13</v>
@@ -4418,19 +4409,19 @@
     </row>
     <row r="70" spans="1:9" ht="16">
       <c r="A70" s="17" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C70" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D70" s="42" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F70" s="19">
         <v>2023</v>
@@ -4439,7 +4430,7 @@
         <v>2040</v>
       </c>
       <c r="H70" s="18" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="I70" s="6" t="s">
         <v>13</v>
@@ -4447,19 +4438,19 @@
     </row>
     <row r="71" spans="1:9" ht="16">
       <c r="A71" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D71" s="9" t="s">
         <v>251</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="E71" s="9" t="s">
         <v>252</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D71" s="9" t="s">
-        <v>253</v>
-      </c>
-      <c r="E71" s="9" t="s">
-        <v>254</v>
       </c>
       <c r="F71" s="2">
         <v>2011</v>
@@ -4473,19 +4464,19 @@
     </row>
     <row r="72" spans="1:9" ht="16">
       <c r="A72" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D72" s="9" t="s">
         <v>255</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="E72" s="45" t="s">
         <v>256</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D72" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="E72" s="45" t="s">
-        <v>258</v>
       </c>
       <c r="F72" s="2">
         <v>2014</v>
@@ -4499,19 +4490,19 @@
     </row>
     <row r="73" spans="1:9" ht="16">
       <c r="A73" s="17" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C73" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D73" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E73" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F73" s="19">
         <v>2022</v>
@@ -4520,7 +4511,7 @@
         <v>2039</v>
       </c>
       <c r="H73" s="18" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="I73" s="6" t="s">
         <v>13</v>
@@ -4528,19 +4519,19 @@
     </row>
     <row r="74" spans="1:9" ht="16">
       <c r="A74" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D74" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="E74" s="45" t="s">
         <v>263</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D74" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="E74" s="45" t="s">
-        <v>265</v>
       </c>
       <c r="F74" s="2">
         <v>2012</v>
@@ -4549,7 +4540,7 @@
         <v>2029</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="I74" s="6" t="s">
         <v>83</v>
@@ -4557,19 +4548,19 @@
     </row>
     <row r="75" spans="1:9" ht="16">
       <c r="A75" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D75" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="E75" s="9" t="s">
         <v>268</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="E75" s="9" t="s">
-        <v>270</v>
       </c>
       <c r="F75" s="2">
         <v>2001</v>
@@ -4583,19 +4574,19 @@
     </row>
     <row r="76" spans="1:9" ht="16">
       <c r="A76" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E76" s="9" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F76" s="2">
         <v>2016</v>
@@ -4604,7 +4595,7 @@
         <v>2036</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I76" s="6" t="s">
         <v>83</v>
@@ -4612,19 +4603,19 @@
     </row>
     <row r="77" spans="1:9" ht="16">
       <c r="A77" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D77" s="9" t="s">
         <v>274</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="E77" s="9" t="s">
         <v>275</v>
-      </c>
-      <c r="C77" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>276</v>
-      </c>
-      <c r="E77" s="9" t="s">
-        <v>277</v>
       </c>
       <c r="F77" s="2">
         <v>2006</v>
@@ -4638,19 +4629,19 @@
     </row>
     <row r="78" spans="1:9" ht="16">
       <c r="A78" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D78" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="E78" s="45" t="s">
         <v>279</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D78" s="9" t="s">
-        <v>280</v>
-      </c>
-      <c r="E78" s="45" t="s">
-        <v>281</v>
       </c>
       <c r="F78" s="2">
         <v>2021</v>
@@ -4664,19 +4655,19 @@
     </row>
     <row r="79" spans="1:9" ht="16">
       <c r="A79" s="17" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B79" s="17" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C79" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D79" s="42" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="E79" s="47" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="F79" s="19">
         <v>2011</v>
@@ -4685,7 +4676,7 @@
         <v>2031</v>
       </c>
       <c r="H79" s="18" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I79" s="6" t="s">
         <v>13</v>
@@ -4693,19 +4684,19 @@
     </row>
     <row r="80" spans="1:9" ht="16">
       <c r="A80" s="17" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C80" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D80" s="42" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="E80" s="47" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="F80" s="19">
         <v>2011</v>
@@ -4714,7 +4705,7 @@
         <v>2031</v>
       </c>
       <c r="H80" s="18" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I80" s="6" t="s">
         <v>13</v>
@@ -4722,19 +4713,19 @@
     </row>
     <row r="81" spans="1:9" ht="16">
       <c r="A81" s="17" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C81" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D81" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E81" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F81" s="19">
         <v>2022</v>
@@ -4743,7 +4734,7 @@
         <v>2039</v>
       </c>
       <c r="H81" s="18" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I81" s="6" t="s">
         <v>13</v>
@@ -4751,19 +4742,19 @@
     </row>
     <row r="82" spans="1:9" ht="16">
       <c r="A82" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D82" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="B82" s="1" t="s">
+      <c r="E82" s="45" t="s">
         <v>292</v>
-      </c>
-      <c r="C82" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D82" s="9" t="s">
-        <v>293</v>
-      </c>
-      <c r="E82" s="45" t="s">
-        <v>294</v>
       </c>
       <c r="F82" s="2">
         <v>2011</v>
@@ -4777,19 +4768,19 @@
     </row>
     <row r="83" spans="1:9" ht="16">
       <c r="A83" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D83" s="45" t="s">
         <v>295</v>
       </c>
-      <c r="B83" s="1" t="s">
+      <c r="E83" s="9" t="s">
         <v>296</v>
-      </c>
-      <c r="C83" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D83" s="45" t="s">
-        <v>297</v>
-      </c>
-      <c r="E83" s="9" t="s">
-        <v>298</v>
       </c>
       <c r="F83" s="2">
         <v>2010</v>
@@ -4803,19 +4794,19 @@
     </row>
     <row r="84" spans="1:9" ht="16">
       <c r="A84" s="17" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C84" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D84" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E84" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F84" s="19">
         <v>2022</v>
@@ -4824,7 +4815,7 @@
         <v>2039</v>
       </c>
       <c r="H84" s="18" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="I84" s="6" t="s">
         <v>13</v>
@@ -4832,19 +4823,19 @@
     </row>
     <row r="85" spans="1:9" ht="16">
       <c r="A85" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D85" s="9" t="s">
         <v>302</v>
       </c>
-      <c r="B85" s="1" t="s">
+      <c r="E85" s="9" t="s">
         <v>303</v>
-      </c>
-      <c r="C85" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D85" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="E85" s="9" t="s">
-        <v>305</v>
       </c>
       <c r="F85" s="2">
         <v>2011</v>
@@ -4858,19 +4849,19 @@
     </row>
     <row r="86" spans="1:9" ht="16">
       <c r="A86" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D86" s="9" t="s">
         <v>306</v>
       </c>
-      <c r="B86" s="1" t="s">
+      <c r="E86" s="45" t="s">
         <v>307</v>
-      </c>
-      <c r="C86" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D86" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="E86" s="45" t="s">
-        <v>309</v>
       </c>
       <c r="F86" s="2">
         <v>2012</v>
@@ -4884,19 +4875,19 @@
     </row>
     <row r="87" spans="1:9" ht="16">
       <c r="A87" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="B87" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C87" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D87" s="42" t="s">
         <v>310</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="E87" s="42" t="s">
         <v>311</v>
-      </c>
-      <c r="C87" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="D87" s="42" t="s">
-        <v>312</v>
-      </c>
-      <c r="E87" s="42" t="s">
-        <v>313</v>
       </c>
       <c r="F87" s="19">
         <v>2008</v>
@@ -4905,7 +4896,7 @@
         <v>2028</v>
       </c>
       <c r="H87" s="18" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="I87" s="6" t="s">
         <v>13</v>
@@ -4913,19 +4904,19 @@
     </row>
     <row r="88" spans="1:9" ht="16">
       <c r="A88" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D88" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="B88" s="1" t="s">
+      <c r="E88" s="9" t="s">
         <v>316</v>
-      </c>
-      <c r="C88" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D88" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="E88" s="9" t="s">
-        <v>318</v>
       </c>
       <c r="F88" s="2">
         <v>2006</v>
@@ -4939,19 +4930,19 @@
     </row>
     <row r="89" spans="1:9" ht="16">
       <c r="A89" s="17" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B89" s="17" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="C89" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D89" s="42" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E89" s="42" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="F89" s="19">
         <v>1994</v>
@@ -4960,7 +4951,7 @@
         <v>2025</v>
       </c>
       <c r="H89" s="18" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="I89" s="6" t="s">
         <v>13</v>
@@ -4968,19 +4959,19 @@
     </row>
     <row r="90" spans="1:9" ht="16">
       <c r="A90" s="17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C90" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D90" s="42" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="E90" s="42" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="F90" s="19">
         <v>2011</v>
@@ -4989,7 +4980,7 @@
         <v>2026</v>
       </c>
       <c r="H90" s="18" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="I90" s="6" t="s">
         <v>13</v>
@@ -4997,19 +4988,19 @@
     </row>
     <row r="91" spans="1:9" ht="16">
       <c r="A91" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="C91" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D91" s="9" t="s">
         <v>325</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="E91" s="9" t="s">
         <v>326</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D91" s="9" t="s">
-        <v>327</v>
-      </c>
-      <c r="E91" s="9" t="s">
-        <v>328</v>
       </c>
       <c r="F91" s="2">
         <v>2011</v>
@@ -5023,19 +5014,19 @@
     </row>
     <row r="92" spans="1:9" ht="16">
       <c r="A92" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D92" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="E92" s="45" t="s">
         <v>330</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D92" s="9" t="s">
-        <v>331</v>
-      </c>
-      <c r="E92" s="45" t="s">
-        <v>332</v>
       </c>
       <c r="F92" s="2">
         <v>2011</v>
@@ -5049,19 +5040,19 @@
     </row>
     <row r="93" spans="1:9" ht="16">
       <c r="A93" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D93" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="E93" s="45" t="s">
         <v>334</v>
-      </c>
-      <c r="C93" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D93" s="9" t="s">
-        <v>335</v>
-      </c>
-      <c r="E93" s="45" t="s">
-        <v>336</v>
       </c>
       <c r="F93" s="2">
         <v>2006</v>
@@ -5075,19 +5066,19 @@
     </row>
     <row r="94" spans="1:9" ht="16">
       <c r="A94" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D94" s="9" t="s">
         <v>337</v>
       </c>
-      <c r="B94" s="1" t="s">
+      <c r="E94" s="9" t="s">
         <v>338</v>
-      </c>
-      <c r="C94" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D94" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="E94" s="9" t="s">
-        <v>340</v>
       </c>
       <c r="F94" s="2">
         <v>2006</v>
@@ -5101,19 +5092,19 @@
     </row>
     <row r="95" spans="1:9" ht="16">
       <c r="A95" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D95" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="B95" s="1" t="s">
+      <c r="E95" s="9" t="s">
         <v>342</v>
-      </c>
-      <c r="C95" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D95" s="9" t="s">
-        <v>343</v>
-      </c>
-      <c r="E95" s="9" t="s">
-        <v>344</v>
       </c>
       <c r="F95" s="2">
         <v>2004</v>
@@ -5127,19 +5118,19 @@
     </row>
     <row r="96" spans="1:9" ht="16">
       <c r="A96" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D96" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="E96" s="9" t="s">
         <v>346</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D96" s="9" t="s">
-        <v>347</v>
-      </c>
-      <c r="E96" s="9" t="s">
-        <v>348</v>
       </c>
       <c r="F96" s="2">
         <v>2006</v>
@@ -5153,19 +5144,19 @@
     </row>
     <row r="97" spans="1:9" ht="16">
       <c r="A97" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D97" s="9" t="s">
         <v>349</v>
       </c>
-      <c r="B97" s="1" t="s">
+      <c r="E97" s="9" t="s">
         <v>350</v>
-      </c>
-      <c r="C97" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D97" s="9" t="s">
-        <v>351</v>
-      </c>
-      <c r="E97" s="9" t="s">
-        <v>352</v>
       </c>
       <c r="F97" s="2">
         <v>2011</v>
@@ -5179,19 +5170,19 @@
     </row>
     <row r="98" spans="1:9" ht="16">
       <c r="A98" s="17" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C98" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D98" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E98" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F98" s="19">
         <v>2022</v>
@@ -5200,7 +5191,7 @@
         <v>2039</v>
       </c>
       <c r="H98" s="18" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="I98" s="6" t="s">
         <v>13</v>
@@ -5208,19 +5199,19 @@
     </row>
     <row r="99" spans="1:9" ht="16">
       <c r="A99" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D99" s="9" t="s">
         <v>356</v>
       </c>
-      <c r="B99" s="1" t="s">
+      <c r="E99" s="45" t="s">
         <v>357</v>
-      </c>
-      <c r="C99" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D99" s="9" t="s">
-        <v>358</v>
-      </c>
-      <c r="E99" s="45" t="s">
-        <v>359</v>
       </c>
       <c r="F99" s="2">
         <v>2015</v>
@@ -5234,19 +5225,19 @@
     </row>
     <row r="100" spans="1:9" ht="16">
       <c r="A100" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D100" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="B100" s="1" t="s">
+      <c r="E100" s="9" t="s">
         <v>361</v>
-      </c>
-      <c r="C100" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D100" s="9" t="s">
-        <v>362</v>
-      </c>
-      <c r="E100" s="9" t="s">
-        <v>363</v>
       </c>
       <c r="F100" s="2">
         <v>2006</v>
@@ -5260,19 +5251,19 @@
     </row>
     <row r="101" spans="1:9" ht="16">
       <c r="A101" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D101" s="9" t="s">
         <v>364</v>
       </c>
-      <c r="B101" s="1" t="s">
+      <c r="E101" s="45" t="s">
         <v>365</v>
-      </c>
-      <c r="C101" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D101" s="9" t="s">
-        <v>366</v>
-      </c>
-      <c r="E101" s="45" t="s">
-        <v>367</v>
       </c>
       <c r="F101" s="2">
         <v>2004</v>
@@ -5286,10 +5277,10 @@
     </row>
     <row r="102" spans="1:9" ht="16">
       <c r="A102" s="27" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B102" s="27" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C102" s="28" t="s">
         <v>11</v>
@@ -5307,7 +5298,7 @@
         <v>11</v>
       </c>
       <c r="H102" s="29" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="I102" s="6" t="s">
         <v>13</v>
@@ -5315,19 +5306,19 @@
     </row>
     <row r="103" spans="1:9" ht="16">
       <c r="A103" s="15" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B103" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="C103" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D103" s="41" t="s">
         <v>369</v>
       </c>
-      <c r="C103" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D103" s="41" t="s">
-        <v>371</v>
-      </c>
       <c r="E103" s="41" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="F103" s="16">
         <v>2006</v>
@@ -5336,7 +5327,7 @@
         <v>2029</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="I103" s="6" t="s">
         <v>13</v>
@@ -5344,19 +5335,19 @@
     </row>
     <row r="104" spans="1:9" ht="16">
       <c r="A104" s="15" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B104" s="15" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C104" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D104" s="41" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="E104" s="41" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F104" s="16">
         <v>2011</v>
@@ -5365,7 +5356,7 @@
         <v>2032</v>
       </c>
       <c r="H104" s="10" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="I104" s="6" t="s">
         <v>13</v>
@@ -5373,19 +5364,19 @@
     </row>
     <row r="105" spans="1:9" ht="16">
       <c r="A105" s="15" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B105" s="15" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C105" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D105" s="41" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E105" s="41" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F105" s="16">
         <v>2012</v>
@@ -5394,7 +5385,7 @@
         <v>2032</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="I105" s="6" t="s">
         <v>13</v>
@@ -5402,19 +5393,19 @@
     </row>
     <row r="106" spans="1:9" ht="16">
       <c r="A106" s="15" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B106" s="15" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C106" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D106" s="41" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E106" s="41" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="F106" s="16">
         <v>2011</v>
@@ -5423,7 +5414,7 @@
         <v>2028</v>
       </c>
       <c r="H106" s="10" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="I106" s="6" t="s">
         <v>13</v>
@@ -5431,19 +5422,19 @@
     </row>
     <row r="107" spans="1:9" ht="16">
       <c r="A107" s="15" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="B107" s="15" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C107" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D107" s="41" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="E107" s="41" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="F107" s="16">
         <v>2006</v>
@@ -5452,7 +5443,7 @@
         <v>2028</v>
       </c>
       <c r="H107" s="10" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="I107" s="6" t="s">
         <v>13</v>
@@ -5460,19 +5451,19 @@
     </row>
     <row r="108" spans="1:9" ht="16">
       <c r="A108" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D108" s="9" t="s">
         <v>385</v>
       </c>
-      <c r="B108" s="1" t="s">
+      <c r="E108" s="9" t="s">
         <v>386</v>
-      </c>
-      <c r="C108" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D108" s="9" t="s">
-        <v>387</v>
-      </c>
-      <c r="E108" s="9" t="s">
-        <v>388</v>
       </c>
       <c r="F108" s="2">
         <v>2011</v>
@@ -5486,19 +5477,19 @@
     </row>
     <row r="109" spans="1:9" ht="16">
       <c r="A109" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D109" s="9" t="s">
         <v>389</v>
       </c>
-      <c r="B109" s="1" t="s">
+      <c r="E109" s="9" t="s">
         <v>390</v>
-      </c>
-      <c r="C109" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D109" s="9" t="s">
-        <v>391</v>
-      </c>
-      <c r="E109" s="9" t="s">
-        <v>392</v>
       </c>
       <c r="F109" s="2">
         <v>2006</v>
@@ -5512,19 +5503,19 @@
     </row>
     <row r="110" spans="1:9" ht="16">
       <c r="A110" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D110" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="B110" s="1" t="s">
+      <c r="E110" s="9" t="s">
         <v>394</v>
-      </c>
-      <c r="C110" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D110" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="E110" s="9" t="s">
-        <v>396</v>
       </c>
       <c r="F110" s="2">
         <v>2013</v>
@@ -5538,19 +5529,19 @@
     </row>
     <row r="111" spans="1:9" ht="16">
       <c r="A111" s="17" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="B111" s="17" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="C111" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D111" s="42" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="E111" s="42" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="F111" s="19">
         <v>2011</v>
@@ -5559,7 +5550,7 @@
         <v>2031</v>
       </c>
       <c r="H111" s="18" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="I111" s="6" t="s">
         <v>13</v>
@@ -5567,19 +5558,19 @@
     </row>
     <row r="112" spans="1:9" ht="16">
       <c r="A112" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D112" s="9" t="s">
         <v>400</v>
       </c>
-      <c r="B112" s="1" t="s">
+      <c r="E112" s="9" t="s">
         <v>401</v>
-      </c>
-      <c r="C112" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D112" s="9" t="s">
-        <v>402</v>
-      </c>
-      <c r="E112" s="9" t="s">
-        <v>403</v>
       </c>
       <c r="F112" s="2">
         <v>2001</v>
@@ -5593,19 +5584,19 @@
     </row>
     <row r="113" spans="1:9" ht="16">
       <c r="A113" s="17" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="B113" s="17" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C113" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D113" s="42" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="E113" s="42" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="F113" s="19">
         <v>2022</v>
@@ -5614,7 +5605,7 @@
         <v>2039</v>
       </c>
       <c r="H113" s="18" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="I113" s="6" t="s">
         <v>13</v>
@@ -5622,19 +5613,19 @@
     </row>
     <row r="114" spans="1:9" ht="16">
       <c r="A114" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D114" s="9" t="s">
         <v>407</v>
       </c>
-      <c r="B114" s="1" t="s">
+      <c r="E114" s="9" t="s">
         <v>408</v>
-      </c>
-      <c r="C114" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D114" s="9" t="s">
-        <v>409</v>
-      </c>
-      <c r="E114" s="9" t="s">
-        <v>410</v>
       </c>
       <c r="F114" s="2">
         <v>2006</v>
@@ -5648,19 +5639,19 @@
     </row>
     <row r="115" spans="1:9" ht="16">
       <c r="A115" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="C115" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D115" s="9" t="s">
         <v>411</v>
       </c>
-      <c r="B115" s="1" t="s">
+      <c r="E115" s="9" t="s">
         <v>412</v>
-      </c>
-      <c r="C115" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D115" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="E115" s="9" t="s">
-        <v>414</v>
       </c>
       <c r="F115" s="2">
         <v>2013</v>
@@ -5674,19 +5665,19 @@
     </row>
     <row r="116" spans="1:9" ht="16">
       <c r="A116" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D116" s="9" t="s">
         <v>415</v>
       </c>
-      <c r="B116" s="1" t="s">
+      <c r="E116" s="9" t="s">
         <v>416</v>
-      </c>
-      <c r="C116" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D116" s="9" t="s">
-        <v>417</v>
-      </c>
-      <c r="E116" s="9" t="s">
-        <v>418</v>
       </c>
       <c r="F116" s="2">
         <v>2011</v>
@@ -5700,19 +5691,19 @@
     </row>
     <row r="117" spans="1:9" ht="16">
       <c r="A117" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D117" s="9" t="s">
         <v>419</v>
       </c>
-      <c r="B117" s="1" t="s">
+      <c r="E117" s="24" t="s">
         <v>420</v>
-      </c>
-      <c r="C117" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D117" s="9" t="s">
-        <v>421</v>
-      </c>
-      <c r="E117" s="24" t="s">
-        <v>422</v>
       </c>
       <c r="F117" s="2">
         <v>2011</v>
@@ -5726,19 +5717,19 @@
     </row>
     <row r="118" spans="1:9" ht="16">
       <c r="A118" s="17" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B118" s="17" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C118" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E118" s="40" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F118" s="19">
         <v>2011</v>
@@ -5747,7 +5738,7 @@
         <v>2026</v>
       </c>
       <c r="H118" s="18" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="I118" s="6" t="s">
         <v>13</v>
@@ -5755,19 +5746,19 @@
     </row>
     <row r="119" spans="1:9" ht="16">
       <c r="A119" s="17" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B119" s="17" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C119" s="19" t="s">
         <v>27</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E119" s="40" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F119" s="19">
         <v>2011</v>
@@ -5776,7 +5767,7 @@
         <v>2026</v>
       </c>
       <c r="H119" s="18" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="I119" s="6" t="s">
         <v>13</v>
@@ -5784,19 +5775,19 @@
     </row>
     <row r="120" spans="1:9" ht="16">
       <c r="A120" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D120" s="9" t="s">
         <v>429</v>
       </c>
-      <c r="B120" s="1" t="s">
+      <c r="E120" s="9" t="s">
         <v>430</v>
-      </c>
-      <c r="C120" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D120" s="9" t="s">
-        <v>431</v>
-      </c>
-      <c r="E120" s="9" t="s">
-        <v>432</v>
       </c>
       <c r="F120" s="2">
         <v>2023</v>
@@ -5810,10 +5801,10 @@
     </row>
     <row r="121" spans="1:9" ht="16">
       <c r="A121" s="27" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B121" s="27" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="C121" s="28" t="s">
         <v>11</v>
@@ -5831,7 +5822,7 @@
         <v>11</v>
       </c>
       <c r="H121" s="29" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="I121" s="6" t="s">
         <v>83</v>
@@ -5839,19 +5830,19 @@
     </row>
     <row r="122" spans="1:9" ht="16">
       <c r="A122" s="16" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B122" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="C122" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D122" s="41" t="s">
         <v>434</v>
       </c>
-      <c r="C122" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D122" s="41" t="s">
-        <v>436</v>
-      </c>
       <c r="E122" s="41" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F122" s="16">
         <v>2011</v>
@@ -5860,7 +5851,7 @@
         <v>2029</v>
       </c>
       <c r="H122" s="10" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="I122" s="6" t="s">
         <v>83</v>
@@ -5868,19 +5859,19 @@
     </row>
     <row r="123" spans="1:9" ht="16">
       <c r="A123" s="16" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B123" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="C123" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D123" s="41" t="s">
         <v>434</v>
       </c>
-      <c r="C123" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D123" s="41" t="s">
-        <v>436</v>
-      </c>
       <c r="E123" s="41" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F123" s="16">
         <v>2011</v>
@@ -5889,7 +5880,7 @@
         <v>2029</v>
       </c>
       <c r="H123" s="10" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="I123" s="6" t="s">
         <v>83</v>
@@ -5897,19 +5888,19 @@
     </row>
     <row r="124" spans="1:9" ht="16">
       <c r="A124" s="16" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="B124" s="16" t="s">
+        <v>432</v>
+      </c>
+      <c r="C124" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D124" s="41" t="s">
         <v>434</v>
       </c>
-      <c r="C124" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D124" s="41" t="s">
-        <v>436</v>
-      </c>
       <c r="E124" s="41" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F124" s="16">
         <v>2011</v>
@@ -5918,7 +5909,7 @@
         <v>2029</v>
       </c>
       <c r="H124" s="10" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="I124" s="6" t="s">
         <v>83</v>
@@ -5926,19 +5917,19 @@
     </row>
     <row r="125" spans="1:9" ht="16">
       <c r="A125" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C125" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D125" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="B125" s="1" t="s">
+      <c r="E125" s="9" t="s">
         <v>442</v>
-      </c>
-      <c r="C125" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D125" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="E125" s="9" t="s">
-        <v>444</v>
       </c>
       <c r="F125" s="2">
         <v>2010</v>
@@ -5952,19 +5943,19 @@
     </row>
     <row r="126" spans="1:9" ht="16">
       <c r="A126" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C126" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D126" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="B126" s="1" t="s">
+      <c r="E126" s="9" t="s">
         <v>446</v>
-      </c>
-      <c r="C126" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D126" s="9" t="s">
-        <v>447</v>
-      </c>
-      <c r="E126" s="9" t="s">
-        <v>448</v>
       </c>
       <c r="F126" s="2">
         <v>2006</v>
@@ -5978,19 +5969,19 @@
     </row>
     <row r="127" spans="1:9" ht="16">
       <c r="A127" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="C127" s="6" t="s">
         <v>18</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="E127" s="9" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="F127" s="2">
         <v>2023</v>
@@ -5999,7 +5990,7 @@
         <v>2040</v>
       </c>
       <c r="H127" s="6" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="I127" s="6" t="s">
         <v>83</v>
@@ -6007,19 +5998,19 @@
     </row>
     <row r="128" spans="1:9" ht="16">
       <c r="A128" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C128" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D128" s="9" t="s">
         <v>452</v>
       </c>
-      <c r="B128" s="1" t="s">
+      <c r="E128" s="24" t="s">
         <v>453</v>
-      </c>
-      <c r="C128" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D128" s="9" t="s">
-        <v>454</v>
-      </c>
-      <c r="E128" s="24" t="s">
-        <v>455</v>
       </c>
       <c r="F128" s="2">
         <v>2024</v>
@@ -6033,19 +6024,19 @@
     </row>
     <row r="129" spans="1:9" ht="16">
       <c r="A129" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C129" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D129" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="B129" s="1" t="s">
+      <c r="E129" s="9" t="s">
         <v>457</v>
-      </c>
-      <c r="C129" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D129" s="9" t="s">
-        <v>458</v>
-      </c>
-      <c r="E129" s="9" t="s">
-        <v>459</v>
       </c>
       <c r="F129" s="2">
         <v>2020</v>
@@ -6059,19 +6050,19 @@
     </row>
     <row r="130" spans="1:9" ht="16">
       <c r="A130" s="30" t="s">
+        <v>458</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="C130" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D130" s="9" t="s">
         <v>460</v>
       </c>
-      <c r="B130" s="1" t="s">
+      <c r="E130" s="9" t="s">
         <v>461</v>
-      </c>
-      <c r="C130" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D130" s="9" t="s">
-        <v>462</v>
-      </c>
-      <c r="E130" s="9" t="s">
-        <v>463</v>
       </c>
       <c r="F130" s="2">
         <v>2015</v>
@@ -6085,19 +6076,19 @@
     </row>
     <row r="131" spans="1:9" ht="16">
       <c r="A131" s="30" t="s">
+        <v>462</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C131" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D131" s="9" t="s">
         <v>464</v>
       </c>
-      <c r="B131" s="1" t="s">
+      <c r="E131" s="9" t="s">
         <v>465</v>
-      </c>
-      <c r="C131" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D131" s="9" t="s">
-        <v>466</v>
-      </c>
-      <c r="E131" s="9" t="s">
-        <v>467</v>
       </c>
       <c r="F131" s="2">
         <v>2015</v>
@@ -6111,19 +6102,19 @@
     </row>
     <row r="132" spans="1:9" ht="16">
       <c r="A132" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="C132" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D132" s="9" t="s">
         <v>468</v>
       </c>
-      <c r="B132" s="1" t="s">
+      <c r="E132" s="9" t="s">
         <v>469</v>
-      </c>
-      <c r="C132" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D132" s="9" t="s">
-        <v>470</v>
-      </c>
-      <c r="E132" s="9" t="s">
-        <v>471</v>
       </c>
       <c r="F132" s="2">
         <v>2016</v>
@@ -6137,19 +6128,19 @@
     </row>
     <row r="133" spans="1:9" ht="16">
       <c r="A133" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C133" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D133" s="9" t="s">
         <v>472</v>
       </c>
-      <c r="B133" s="1" t="s">
+      <c r="E133" s="9" t="s">
         <v>473</v>
-      </c>
-      <c r="C133" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D133" s="9" t="s">
-        <v>474</v>
-      </c>
-      <c r="E133" s="9" t="s">
-        <v>475</v>
       </c>
       <c r="F133" s="2">
         <v>2011</v>
@@ -6163,19 +6154,19 @@
     </row>
     <row r="134" spans="1:9" ht="16">
       <c r="A134" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C134" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D134" s="9" t="s">
         <v>476</v>
       </c>
-      <c r="B134" s="1" t="s">
+      <c r="E134" s="9" t="s">
         <v>477</v>
-      </c>
-      <c r="C134" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D134" s="9" t="s">
-        <v>478</v>
-      </c>
-      <c r="E134" s="9" t="s">
-        <v>479</v>
       </c>
       <c r="F134" s="2">
         <v>2017</v>
@@ -6189,19 +6180,19 @@
     </row>
     <row r="135" spans="1:9" ht="16">
       <c r="A135" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="C135" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D135" s="9" t="s">
         <v>480</v>
       </c>
-      <c r="B135" s="1" t="s">
+      <c r="E135" s="45" t="s">
         <v>481</v>
-      </c>
-      <c r="C135" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D135" s="9" t="s">
-        <v>482</v>
-      </c>
-      <c r="E135" s="45" t="s">
-        <v>483</v>
       </c>
       <c r="F135" s="2">
         <v>2011</v>
@@ -6476,31 +6467,31 @@
         <v>7</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="6" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B9" s="46" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="6" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
     </row>
   </sheetData>
@@ -6547,13 +6538,13 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" s="31" t="s">
+        <v>482</v>
+      </c>
+      <c r="B2" s="32" t="s">
+        <v>483</v>
+      </c>
+      <c r="C2" s="32" t="s">
         <v>484</v>
-      </c>
-      <c r="B2" s="32" t="s">
-        <v>485</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>486</v>
       </c>
       <c r="D2" s="33"/>
       <c r="E2" s="33"/>
@@ -6564,13 +6555,13 @@
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B3" s="32" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="C3" s="32" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
       <c r="D3" s="33"/>
       <c r="E3" s="33"/>
@@ -6582,10 +6573,10 @@
     <row r="4" spans="1:9">
       <c r="A4" s="32"/>
       <c r="B4" s="32" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
       <c r="C4" s="32" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="D4" s="33"/>
       <c r="E4" s="33"/>
@@ -6597,10 +6588,10 @@
     <row r="5" spans="1:9">
       <c r="A5" s="32"/>
       <c r="B5" s="32" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C5" s="32" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="D5" s="33"/>
       <c r="E5" s="33"/>
@@ -6610,13 +6601,13 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B6" s="32" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="C6" s="32" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="D6" s="33"/>
       <c r="E6" s="33"/>
@@ -6627,10 +6618,10 @@
     <row r="7" spans="1:9">
       <c r="A7" s="32"/>
       <c r="B7" s="32" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="C7" s="32" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="D7" s="33"/>
       <c r="E7" s="33"/>
@@ -6642,10 +6633,10 @@
     <row r="8" spans="1:9">
       <c r="A8" s="32"/>
       <c r="B8" s="32" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="C8" s="32" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="33"/>
@@ -6657,10 +6648,10 @@
     <row r="9" spans="1:9">
       <c r="A9" s="32"/>
       <c r="B9" s="32" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="C9" s="32" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="D9" s="33"/>
       <c r="E9" s="33"/>
@@ -6672,10 +6663,10 @@
     <row r="10" spans="1:9">
       <c r="A10" s="32"/>
       <c r="B10" s="32" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="C10" s="32" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="D10" s="33"/>
       <c r="E10" s="33"/>
@@ -6686,10 +6677,10 @@
     <row r="11" spans="1:9">
       <c r="A11" s="32"/>
       <c r="B11" s="32" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="C11" s="32" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="D11" s="33"/>
       <c r="E11" s="33"/>
@@ -6700,10 +6691,10 @@
     <row r="12" spans="1:9">
       <c r="A12" s="32"/>
       <c r="B12" s="32" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C12" s="32" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="D12" s="33"/>
       <c r="E12" s="33"/>
@@ -6713,13 +6704,13 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="35" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B13" s="36" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C13" s="36" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="D13" s="35"/>
       <c r="E13" s="36"/>
@@ -6729,13 +6720,13 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="35" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B14" s="36" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="C14" s="36" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="D14" s="35"/>
       <c r="E14" s="36"/>
@@ -6746,13 +6737,13 @@
     <row r="15" spans="1:9">
       <c r="A15" s="32"/>
       <c r="B15" s="32" t="s">
+        <v>509</v>
+      </c>
+      <c r="C15" s="32" t="s">
+        <v>510</v>
+      </c>
+      <c r="D15" s="31" t="s">
         <v>511</v>
-      </c>
-      <c r="C15" s="32" t="s">
-        <v>512</v>
-      </c>
-      <c r="D15" s="31" t="s">
-        <v>513</v>
       </c>
       <c r="E15" s="33"/>
       <c r="F15" s="33"/>
@@ -6762,10 +6753,10 @@
     <row r="16" spans="1:9">
       <c r="A16" s="32"/>
       <c r="B16" s="32" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C16" s="32" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D16" s="33"/>
       <c r="E16" s="33"/>
@@ -6776,10 +6767,10 @@
     <row r="17" spans="1:29">
       <c r="A17" s="32"/>
       <c r="B17" s="32" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C17" s="32" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D17" s="33"/>
       <c r="E17" s="33"/>
@@ -6790,13 +6781,13 @@
     <row r="18" spans="1:29">
       <c r="A18" s="32"/>
       <c r="B18" s="32" t="s">
+        <v>516</v>
+      </c>
+      <c r="C18" s="32" t="s">
+        <v>517</v>
+      </c>
+      <c r="D18" s="31" t="s">
         <v>518</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>519</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>520</v>
       </c>
       <c r="E18" s="33"/>
       <c r="F18" s="33"/>
@@ -6806,10 +6797,10 @@
     <row r="19" spans="1:29">
       <c r="A19" s="32"/>
       <c r="B19" s="32" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="C19" s="32" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="D19" s="33"/>
       <c r="E19" s="33"/>
@@ -6820,10 +6811,10 @@
     <row r="20" spans="1:29">
       <c r="A20" s="32"/>
       <c r="B20" s="32" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="C20" s="32" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="D20" s="33"/>
       <c r="E20" s="33"/>
@@ -6834,10 +6825,10 @@
     <row r="21" spans="1:29">
       <c r="A21" s="32"/>
       <c r="B21" s="32" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="C21" s="32" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="D21" s="33"/>
       <c r="E21" s="33"/>
@@ -6848,10 +6839,10 @@
     <row r="22" spans="1:29">
       <c r="A22" s="32"/>
       <c r="B22" s="32" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="C22" s="32" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="D22" s="33"/>
       <c r="E22" s="33"/>
@@ -6862,10 +6853,10 @@
     <row r="23" spans="1:29">
       <c r="A23" s="32"/>
       <c r="B23" s="32" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="C23" s="32" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="D23" s="33"/>
       <c r="E23" s="33"/>
@@ -6897,10 +6888,10 @@
     <row r="24" spans="1:29">
       <c r="A24" s="32"/>
       <c r="B24" s="32" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="C24" s="32" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="D24" s="33"/>
       <c r="E24" s="33"/>
@@ -6931,13 +6922,13 @@
     </row>
     <row r="25" spans="1:29">
       <c r="A25" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B25" s="32" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="C25" s="32" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="D25" s="33"/>
       <c r="E25" s="33"/>
@@ -6968,13 +6959,13 @@
     </row>
     <row r="26" spans="1:29">
       <c r="A26" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B26" s="32" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="C26" s="32" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="D26" s="33"/>
       <c r="E26" s="33"/>
@@ -7005,13 +6996,13 @@
     </row>
     <row r="27" spans="1:29">
       <c r="A27" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B27" s="32" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="C27" s="32" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="D27" s="33"/>
       <c r="E27" s="33"/>
@@ -7042,13 +7033,13 @@
     </row>
     <row r="28" spans="1:29">
       <c r="A28" s="31" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="B28" s="32" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="C28" s="32" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="D28" s="33"/>
       <c r="E28" s="33"/>
@@ -7080,10 +7071,10 @@
     <row r="29" spans="1:29">
       <c r="A29" s="32"/>
       <c r="B29" s="32" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="C29" s="32" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="D29" s="33"/>
       <c r="E29" s="33"/>
@@ -7115,10 +7106,10 @@
     <row r="30" spans="1:29">
       <c r="A30" s="32"/>
       <c r="B30" s="32" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="C30" s="32" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="D30" s="33"/>
       <c r="E30" s="33"/>
@@ -7150,10 +7141,10 @@
     <row r="31" spans="1:29">
       <c r="A31" s="32"/>
       <c r="B31" s="32" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="C31" s="32" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="D31" s="33"/>
       <c r="E31" s="33"/>
@@ -7185,10 +7176,10 @@
     <row r="32" spans="1:29">
       <c r="A32" s="32"/>
       <c r="B32" s="32" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="C32" s="32" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="D32" s="33"/>
       <c r="E32" s="33"/>
@@ -7220,10 +7211,10 @@
     <row r="33" spans="1:29">
       <c r="A33" s="36"/>
       <c r="B33" s="36" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="C33" s="36" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="D33" s="35"/>
       <c r="E33" s="36"/>
@@ -7233,10 +7224,10 @@
     <row r="34" spans="1:29">
       <c r="A34" s="36"/>
       <c r="B34" s="36" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="C34" s="36" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="D34" s="35"/>
       <c r="E34" s="1"/>
@@ -7246,10 +7237,10 @@
     <row r="35" spans="1:29">
       <c r="A35" s="32"/>
       <c r="B35" s="32" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="C35" s="32" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="D35" s="33"/>
       <c r="E35" s="33"/>
@@ -7281,10 +7272,10 @@
     <row r="36" spans="1:29">
       <c r="A36" s="32"/>
       <c r="B36" s="32" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
       <c r="C36" s="32" t="s">
-        <v>556</v>
+        <v>554</v>
       </c>
       <c r="D36" s="33"/>
       <c r="E36" s="33"/>
@@ -7316,10 +7307,10 @@
     <row r="37" spans="1:29">
       <c r="A37" s="36"/>
       <c r="B37" s="36" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C37" s="36" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="D37" s="35"/>
       <c r="E37" s="1"/>
@@ -7329,10 +7320,10 @@
     <row r="38" spans="1:29">
       <c r="A38" s="36"/>
       <c r="B38" s="36" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C38" s="36" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D38" s="35"/>
       <c r="E38" s="1"/>
@@ -7342,10 +7333,10 @@
     <row r="39" spans="1:29">
       <c r="A39" s="36"/>
       <c r="B39" s="36" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C39" s="36" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="D39" s="36"/>
       <c r="E39" s="1"/>
@@ -7355,10 +7346,10 @@
     <row r="40" spans="1:29">
       <c r="A40" s="32"/>
       <c r="B40" s="32" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C40" s="32" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D40" s="33"/>
       <c r="E40" s="34"/>
@@ -7390,10 +7381,10 @@
     <row r="41" spans="1:29">
       <c r="A41" s="32"/>
       <c r="B41" s="32" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C41" s="32" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D41" s="31"/>
       <c r="E41" s="34"/>
@@ -7425,13 +7416,13 @@
     <row r="42" spans="1:29">
       <c r="A42" s="36"/>
       <c r="B42" s="36" t="s">
+        <v>565</v>
+      </c>
+      <c r="C42" s="36" t="s">
+        <v>566</v>
+      </c>
+      <c r="D42" s="35" t="s">
         <v>567</v>
-      </c>
-      <c r="C42" s="36" t="s">
-        <v>568</v>
-      </c>
-      <c r="D42" s="35" t="s">
-        <v>569</v>
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
@@ -7440,13 +7431,13 @@
     <row r="43" spans="1:29">
       <c r="A43" s="37"/>
       <c r="B43" s="38" t="s">
+        <v>568</v>
+      </c>
+      <c r="C43" s="38" t="s">
+        <v>569</v>
+      </c>
+      <c r="D43" s="39" t="s">
         <v>570</v>
-      </c>
-      <c r="C43" s="38" t="s">
-        <v>571</v>
-      </c>
-      <c r="D43" s="39" t="s">
-        <v>572</v>
       </c>
       <c r="E43" s="1"/>
       <c r="F43" s="1"/>

</xml_diff>

<commit_message>
Fifth batch of manually scraped adopted plans
</commit_message>
<xml_diff>
--- a/data/manually_scraped_adopted_plans.xlsx
+++ b/data/manually_scraped_adopted_plans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sianteesdale/Documents/GitHub/local-plan-extractor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB11815-EDE9-2D42-A568-4C01F0A4E9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844DB5CF-60B0-A74C-850C-6424A93725D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35800" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1893,9 +1893,6 @@
     <t>https://www.stalbans.gov.uk/current-local-plan</t>
   </si>
   <si>
-    <t>https://www.stalbans.gov.uk/sites/default/files/documents/publications/planning-building-control/district-local-plan-review-1994/District Local Plan Review 1994 Saved and Deleted Policies Version %5BJuly 2020%5D.pdf</t>
-  </si>
-  <si>
     <t>https://www.sandwell.gov.uk/downloads/download/347/black-country-core-strategy</t>
   </si>
   <si>
@@ -1969,6 +1966,9 @@
   </si>
   <si>
     <t>https://lbhounslow.sharepoint.com/:b:/s/InternetLinks/pp/EcHMd2lpx5xFlwDbyfEsUrcBvxzfTSoTrW3yOphnXdPQzg?e=fsgeqV</t>
+  </si>
+  <si>
+    <t>https://www.stalbans.gov.uk/sites/default/files/documents/publications/planning-building-control/district-local-plan-review-1994/District%20Local%20Plan%20Review%201994%20Saved%20and%20Deleted%20Policies%20Version%20%5BJuly%202020%5D.pdf</t>
   </si>
 </sst>
 </file>
@@ -2573,7 +2573,7 @@
         <v>577</v>
       </c>
       <c r="E5" s="40" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="F5" s="2">
         <v>2023</v>
@@ -2802,7 +2802,7 @@
         <v>588</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F12" s="2">
         <v>2017</v>
@@ -3063,7 +3063,7 @@
         <v>600</v>
       </c>
       <c r="E21" s="40" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="F21" s="2">
         <v>2015</v>
@@ -3092,7 +3092,7 @@
         <v>601</v>
       </c>
       <c r="E22" s="40" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="F22" s="22">
         <v>2011</v>
@@ -3179,7 +3179,7 @@
         <v>606</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="F25" s="2">
         <v>2015</v>
@@ -3330,7 +3330,7 @@
         <v>83</v>
       </c>
       <c r="Q30" s="46" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="16">
@@ -3790,7 +3790,7 @@
         <v>609</v>
       </c>
       <c r="E47" s="47" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="F47" s="19">
         <v>2011</v>
@@ -3958,7 +3958,7 @@
         <v>179</v>
       </c>
       <c r="E53" s="40" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="F53" s="19">
         <v>2011</v>
@@ -3987,7 +3987,7 @@
         <v>610</v>
       </c>
       <c r="E54" s="40" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="F54" s="19">
         <v>2011</v>
@@ -4259,7 +4259,7 @@
         <v>225</v>
       </c>
       <c r="E64" s="40" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="F64" s="2">
         <v>2015</v>
@@ -4421,7 +4421,7 @@
         <v>613</v>
       </c>
       <c r="E70" s="47" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F70" s="19">
         <v>2023</v>
@@ -4667,7 +4667,7 @@
         <v>616</v>
       </c>
       <c r="E79" s="47" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F79" s="19">
         <v>2011</v>
@@ -4696,7 +4696,7 @@
         <v>617</v>
       </c>
       <c r="E80" s="47" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="F80" s="19">
         <v>2011</v>
@@ -4941,8 +4941,8 @@
       <c r="D89" s="42" t="s">
         <v>618</v>
       </c>
-      <c r="E89" s="42" t="s">
-        <v>619</v>
+      <c r="E89" s="47" t="s">
+        <v>644</v>
       </c>
       <c r="F89" s="19">
         <v>1994</v>
@@ -4968,10 +4968,10 @@
         <v>27</v>
       </c>
       <c r="D90" s="42" t="s">
+        <v>619</v>
+      </c>
+      <c r="E90" s="42" t="s">
         <v>620</v>
-      </c>
-      <c r="E90" s="42" t="s">
-        <v>621</v>
       </c>
       <c r="F90" s="19">
         <v>2011</v>
@@ -5538,10 +5538,10 @@
         <v>27</v>
       </c>
       <c r="D111" s="42" t="s">
+        <v>621</v>
+      </c>
+      <c r="E111" s="42" t="s">
         <v>622</v>
-      </c>
-      <c r="E111" s="42" t="s">
-        <v>623</v>
       </c>
       <c r="F111" s="19">
         <v>2011</v>
@@ -5726,10 +5726,10 @@
         <v>27</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E118" s="40" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F118" s="19">
         <v>2011</v>
@@ -5755,10 +5755,10 @@
         <v>27</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="E119" s="40" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="F119" s="19">
         <v>2011</v>
@@ -6399,6 +6399,7 @@
     <hyperlink ref="E21" r:id="rId191" display="https://centralbedfordshirecouncil.sharepoint.com/sites/Communications/Website and intranet/Forms/AllItems.aspx?id=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2FCentral%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2Epdf&amp;parent=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035&amp;p=true&amp;ga=1" xr:uid="{0A21C8F8-F7E2-ED4D-B000-E3B6AB33E60B}"/>
     <hyperlink ref="D21" r:id="rId192" xr:uid="{F1D92A59-16C4-1E43-9906-76DB10045477}"/>
     <hyperlink ref="E25" r:id="rId193" xr:uid="{B606F106-13F9-3143-9FAD-49CDAA46AED7}"/>
+    <hyperlink ref="E89" r:id="rId194" xr:uid="{719BCB44-5A56-8D4C-92E6-411FB3FF9320}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -6467,31 +6468,31 @@
         <v>7</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="B9" s="46" t="s">
         <v>626</v>
-      </c>
-      <c r="B9" s="46" t="s">
-        <v>627</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>628</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>629</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>630</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Seventh batch of manually scraped adopted plans
</commit_message>
<xml_diff>
--- a/data/manually_scraped_adopted_plans.xlsx
+++ b/data/manually_scraped_adopted_plans.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sianteesdale/Documents/GitHub/local-plan-extractor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844DB5CF-60B0-A74C-850C-6424A93725D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28313B9-7C59-6044-B669-9EDF60B1801A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35800" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="manual-search" sheetId="1" r:id="rId1"/>
-    <sheet name="key" sheetId="3" r:id="rId2"/>
-    <sheet name="Local plans already scraped - i" sheetId="2" r:id="rId3"/>
+    <sheet name="manual-search" sheetId="4" r:id="rId1"/>
+    <sheet name="manual-search-original" sheetId="1" r:id="rId2"/>
+    <sheet name="key" sheetId="3" r:id="rId3"/>
+    <sheet name="Local plans already scraped - i" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1025" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1937" uniqueCount="689">
   <si>
     <t>organisation</t>
   </si>
@@ -1969,6 +1970,138 @@
   </si>
   <si>
     <t>https://www.stalbans.gov.uk/sites/default/files/documents/publications/planning-building-control/district-local-plan-review-1994/District%20Local%20Plan%20Review%201994%20Saved%20and%20Deleted%20Policies%20Version%20%5BJuly%202020%5D.pdf</t>
+  </si>
+  <si>
+    <t>local-authority:BMH</t>
+  </si>
+  <si>
+    <t>Bournemouth Borough Council</t>
+  </si>
+  <si>
+    <t>local-authority:CHC</t>
+  </si>
+  <si>
+    <t>Christchurch Borough Council</t>
+  </si>
+  <si>
+    <t>local-authority:EDO</t>
+  </si>
+  <si>
+    <t>East Dorset District Council</t>
+  </si>
+  <si>
+    <t>local-authority:POL</t>
+  </si>
+  <si>
+    <t>Borough of Poole</t>
+  </si>
+  <si>
+    <t>local-authority:AYL</t>
+  </si>
+  <si>
+    <t>Aylesbury Vale Council</t>
+  </si>
+  <si>
+    <t>local-authority:CHN</t>
+  </si>
+  <si>
+    <t>Chiltern District Council</t>
+  </si>
+  <si>
+    <t>local-authority:SBU</t>
+  </si>
+  <si>
+    <t>South Bucks District Council</t>
+  </si>
+  <si>
+    <t>local-authority:WYO</t>
+  </si>
+  <si>
+    <t>Wycombe District Council</t>
+  </si>
+  <si>
+    <t>local-authority:WEY</t>
+  </si>
+  <si>
+    <t>Weymouth and Portland Borough Council</t>
+  </si>
+  <si>
+    <t>local-authority:WDO</t>
+  </si>
+  <si>
+    <t>West Dorset District Council</t>
+  </si>
+  <si>
+    <t>local-authority:PUR</t>
+  </si>
+  <si>
+    <t>Purbeck District Council</t>
+  </si>
+  <si>
+    <t>local-authority:NDO</t>
+  </si>
+  <si>
+    <t>North Dorset District Council</t>
+  </si>
+  <si>
+    <t>local-authority:SUF</t>
+  </si>
+  <si>
+    <t>Suffolk Coastal District Council</t>
+  </si>
+  <si>
+    <t>local-authority:WAV</t>
+  </si>
+  <si>
+    <t>Waveney District Council</t>
+  </si>
+  <si>
+    <t>local-authority:MEN</t>
+  </si>
+  <si>
+    <t>Mendip District Council</t>
+  </si>
+  <si>
+    <t>local-authority:SEG</t>
+  </si>
+  <si>
+    <t>Sedgemoor District Council</t>
+  </si>
+  <si>
+    <t>local-authority:WSO</t>
+  </si>
+  <si>
+    <t>West Somerset District Council</t>
+  </si>
+  <si>
+    <t>local-authority:TAU</t>
+  </si>
+  <si>
+    <t>Taunton Deane Borough Council</t>
+  </si>
+  <si>
+    <t>local-authority:SSO</t>
+  </si>
+  <si>
+    <t>South Somerset District Council</t>
+  </si>
+  <si>
+    <t>local-authority:DAV</t>
+  </si>
+  <si>
+    <t>Daventry District Council</t>
+  </si>
+  <si>
+    <t>local-authority:NOR</t>
+  </si>
+  <si>
+    <t>Northampton Borough Council</t>
+  </si>
+  <si>
+    <t>local-authority:SNR</t>
+  </si>
+  <si>
+    <t>South Northamptonshire Council</t>
   </si>
 </sst>
 </file>
@@ -2413,6 +2546,4062 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20320CE1-4F34-8F47-ADE2-62B48A867073}">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <dimension ref="A1:Q137"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="22.33203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" customWidth="1"/>
+    <col min="5" max="5" width="14.33203125" customWidth="1"/>
+    <col min="6" max="6" width="11.83203125" customWidth="1"/>
+    <col min="8" max="8" width="45.5" customWidth="1"/>
+    <col min="10" max="10" width="7" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="16">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>572</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="16">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+    </row>
+    <row r="3" spans="1:15" ht="16">
+      <c r="A3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>573</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>574</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2022</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2040</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="7"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+    </row>
+    <row r="4" spans="1:15" ht="16">
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>576</v>
+      </c>
+      <c r="F4" s="2">
+        <v>2023</v>
+      </c>
+      <c r="G4" s="6">
+        <v>2040</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="7"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+    </row>
+    <row r="5" spans="1:15" ht="16">
+      <c r="A5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>577</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>631</v>
+      </c>
+      <c r="F5" s="2">
+        <v>2023</v>
+      </c>
+      <c r="G5" s="2">
+        <v>2029</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="7"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+    </row>
+    <row r="6" spans="1:15" ht="16" hidden="1">
+      <c r="A6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>579</v>
+      </c>
+      <c r="F6" s="2">
+        <v>2020</v>
+      </c>
+      <c r="G6" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+    </row>
+    <row r="7" spans="1:15" ht="16">
+      <c r="A7" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="7"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+    </row>
+    <row r="8" spans="1:15" ht="16">
+      <c r="A8" s="15" t="s">
+        <v>645</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>646</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>580</v>
+      </c>
+      <c r="E8" s="41" t="s">
+        <v>581</v>
+      </c>
+      <c r="F8" s="16">
+        <v>2006</v>
+      </c>
+      <c r="G8" s="16">
+        <v>2026</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+    </row>
+    <row r="9" spans="1:15" ht="16">
+      <c r="A9" s="16" t="s">
+        <v>647</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>648</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="41" t="s">
+        <v>582</v>
+      </c>
+      <c r="E9" s="41" t="s">
+        <v>583</v>
+      </c>
+      <c r="F9" s="16">
+        <v>2014</v>
+      </c>
+      <c r="G9" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+    </row>
+    <row r="10" spans="1:15" ht="16">
+      <c r="A10" s="15" t="s">
+        <v>649</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>650</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>582</v>
+      </c>
+      <c r="E10" s="41" t="s">
+        <v>583</v>
+      </c>
+      <c r="F10" s="16">
+        <v>2014</v>
+      </c>
+      <c r="G10" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I10" s="6"/>
+      <c r="J10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+    </row>
+    <row r="11" spans="1:15" ht="16">
+      <c r="A11" s="15" t="s">
+        <v>651</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>652</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="41" t="s">
+        <v>584</v>
+      </c>
+      <c r="E11" s="41" t="s">
+        <v>585</v>
+      </c>
+      <c r="F11" s="16">
+        <v>2018</v>
+      </c>
+      <c r="G11" s="16">
+        <v>2033</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="7"/>
+    </row>
+    <row r="12" spans="1:15" ht="16">
+      <c r="A12" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="42" t="s">
+        <v>586</v>
+      </c>
+      <c r="E12" s="42" t="s">
+        <v>587</v>
+      </c>
+      <c r="F12" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G12" s="19">
+        <v>2033</v>
+      </c>
+      <c r="H12" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="16">
+      <c r="A13" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>588</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>632</v>
+      </c>
+      <c r="F13" s="2">
+        <v>2017</v>
+      </c>
+      <c r="G13" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="16">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>590</v>
+      </c>
+      <c r="F14" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G14" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="16">
+      <c r="A15" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>591</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>592</v>
+      </c>
+      <c r="F15" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G15" s="2">
+        <v>2031</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="16">
+      <c r="A16" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="16">
+      <c r="A17" s="15" t="s">
+        <v>653</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>654</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="41" t="s">
+        <v>593</v>
+      </c>
+      <c r="E17" s="41" t="s">
+        <v>594</v>
+      </c>
+      <c r="F17" s="16">
+        <v>2013</v>
+      </c>
+      <c r="G17" s="16">
+        <v>2033</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="16">
+      <c r="A18" s="15" t="s">
+        <v>655</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>656</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D18" s="41" t="s">
+        <v>593</v>
+      </c>
+      <c r="E18" s="41" t="s">
+        <v>595</v>
+      </c>
+      <c r="F18" s="16">
+        <v>1997</v>
+      </c>
+      <c r="G18" s="16">
+        <v>2025</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="16">
+      <c r="A19" s="15" t="s">
+        <v>657</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>658</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="41" t="s">
+        <v>593</v>
+      </c>
+      <c r="E19" s="41" t="s">
+        <v>596</v>
+      </c>
+      <c r="F19" s="16">
+        <v>1999</v>
+      </c>
+      <c r="G19" s="16">
+        <v>2025</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="16">
+      <c r="A20" s="15" t="s">
+        <v>659</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>660</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>593</v>
+      </c>
+      <c r="E20" s="41" t="s">
+        <v>597</v>
+      </c>
+      <c r="F20" s="16">
+        <v>2019</v>
+      </c>
+      <c r="G20" s="16">
+        <v>2033</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="16">
+      <c r="A21" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>598</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>599</v>
+      </c>
+      <c r="F21" s="2">
+        <v>2012</v>
+      </c>
+      <c r="G21" s="2">
+        <v>2032</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="16">
+      <c r="A22" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" s="40" t="s">
+        <v>600</v>
+      </c>
+      <c r="E22" s="40" t="s">
+        <v>640</v>
+      </c>
+      <c r="F22" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G22" s="2">
+        <v>2035</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="16">
+      <c r="A23" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>601</v>
+      </c>
+      <c r="E23" s="40" t="s">
+        <v>633</v>
+      </c>
+      <c r="F23" s="22">
+        <v>2011</v>
+      </c>
+      <c r="G23" s="22">
+        <v>2028</v>
+      </c>
+      <c r="H23" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="16">
+      <c r="A24" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>602</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>603</v>
+      </c>
+      <c r="F24" s="2">
+        <v>2010</v>
+      </c>
+      <c r="G24" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="16">
+      <c r="A25" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>604</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>605</v>
+      </c>
+      <c r="F25" s="2">
+        <v>2018</v>
+      </c>
+      <c r="G25" s="2">
+        <v>2035</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="16">
+      <c r="A26" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="E26" s="40" t="s">
+        <v>641</v>
+      </c>
+      <c r="F26" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G26" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="16">
+      <c r="A27" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F27" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G27" s="2">
+        <v>2031</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="16">
+      <c r="A28" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F28" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G28" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="16">
+      <c r="A29" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="F29" s="2">
+        <v>2023</v>
+      </c>
+      <c r="G29" s="2">
+        <v>2040</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="16">
+      <c r="A30" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>607</v>
+      </c>
+      <c r="F30" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G30" s="2">
+        <v>2031</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="16">
+      <c r="A31" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F31" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G31" s="2">
+        <v>2036</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="Q31" s="46"/>
+    </row>
+    <row r="32" spans="1:17" ht="16">
+      <c r="A32" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="F32" s="2">
+        <v>2013</v>
+      </c>
+      <c r="G32" s="2">
+        <v>2033</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="16">
+      <c r="A33" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="F33" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G33" s="2">
+        <v>2028</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="16">
+      <c r="A34" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G34" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H34" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="16">
+      <c r="A35" s="16" t="s">
+        <v>661</v>
+      </c>
+      <c r="B35" s="16" t="s">
+        <v>662</v>
+      </c>
+      <c r="C35" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D35" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="E35" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="F35" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G35" s="16">
+        <v>2031</v>
+      </c>
+      <c r="H35" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="16">
+      <c r="A36" s="16" t="s">
+        <v>663</v>
+      </c>
+      <c r="B36" s="16" t="s">
+        <v>664</v>
+      </c>
+      <c r="C36" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="F36" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G36" s="16">
+        <v>2031</v>
+      </c>
+      <c r="H36" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="16">
+      <c r="A37" s="16" t="s">
+        <v>665</v>
+      </c>
+      <c r="B37" s="16" t="s">
+        <v>666</v>
+      </c>
+      <c r="C37" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D37" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="E37" s="41" t="s">
+        <v>116</v>
+      </c>
+      <c r="F37" s="16">
+        <v>2018</v>
+      </c>
+      <c r="G37" s="16">
+        <v>2034</v>
+      </c>
+      <c r="H37" s="26" t="s">
+        <v>117</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="16">
+      <c r="A38" s="16" t="s">
+        <v>667</v>
+      </c>
+      <c r="B38" s="16" t="s">
+        <v>668</v>
+      </c>
+      <c r="C38" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D38" s="41" t="s">
+        <v>118</v>
+      </c>
+      <c r="E38" s="41" t="s">
+        <v>119</v>
+      </c>
+      <c r="F38" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G38" s="16">
+        <v>2031</v>
+      </c>
+      <c r="H38" s="26" t="s">
+        <v>120</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="16">
+      <c r="A39" s="16" t="s">
+        <v>647</v>
+      </c>
+      <c r="B39" s="16" t="s">
+        <v>648</v>
+      </c>
+      <c r="C39" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D39" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="E39" s="41" t="s">
+        <v>122</v>
+      </c>
+      <c r="F39" s="16">
+        <v>2013</v>
+      </c>
+      <c r="G39" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H39" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="I39" s="6"/>
+    </row>
+    <row r="40" spans="1:9" ht="16">
+      <c r="A40" s="16" t="s">
+        <v>649</v>
+      </c>
+      <c r="B40" s="16" t="s">
+        <v>650</v>
+      </c>
+      <c r="C40" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="E40" s="41" t="s">
+        <v>122</v>
+      </c>
+      <c r="F40" s="16">
+        <v>2013</v>
+      </c>
+      <c r="G40" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H40" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="I40" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="16">
+      <c r="A41" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D41" s="42" t="s">
+        <v>608</v>
+      </c>
+      <c r="E41" s="44" t="s">
+        <v>126</v>
+      </c>
+      <c r="F41" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G41" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H41" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="16">
+      <c r="A42" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D42" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="F42" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G42" s="2">
+        <v>2036</v>
+      </c>
+      <c r="I42" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="16">
+      <c r="A43" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="F43" s="2">
+        <v>2013</v>
+      </c>
+      <c r="G43" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I43" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="16">
+      <c r="A44" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F44" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G44" s="2">
+        <v>2028</v>
+      </c>
+      <c r="H44" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="16">
+      <c r="A45" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F45" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G45" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="16">
+      <c r="A46" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="F46" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G46" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="16">
+      <c r="A47" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F47" s="2">
+        <v>2010</v>
+      </c>
+      <c r="G47" s="2">
+        <v>2025</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="16">
+      <c r="A48" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="F48" s="2">
+        <v>2007</v>
+      </c>
+      <c r="G48" s="2">
+        <v>2022</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="16">
+      <c r="A49" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D49" s="42" t="s">
+        <v>609</v>
+      </c>
+      <c r="E49" s="47" t="s">
+        <v>634</v>
+      </c>
+      <c r="F49" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G49" s="19">
+        <v>2028</v>
+      </c>
+      <c r="H49" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="I49" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="16">
+      <c r="A50" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F50" s="2">
+        <v>2020</v>
+      </c>
+      <c r="G50" s="2">
+        <v>2039</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="16">
+      <c r="A51" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="B51" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H51" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="16">
+      <c r="A52" s="16" t="s">
+        <v>669</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>670</v>
+      </c>
+      <c r="C52" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="E52" s="41" t="s">
+        <v>169</v>
+      </c>
+      <c r="F52" s="16">
+        <v>2018</v>
+      </c>
+      <c r="G52" s="16">
+        <v>2036</v>
+      </c>
+      <c r="H52" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="16">
+      <c r="A53" s="16" t="s">
+        <v>671</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>672</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D53" s="41" t="s">
+        <v>168</v>
+      </c>
+      <c r="E53" s="41" t="s">
+        <v>171</v>
+      </c>
+      <c r="F53" s="16">
+        <v>2014</v>
+      </c>
+      <c r="G53" s="16">
+        <v>2036</v>
+      </c>
+      <c r="H53" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="16">
+      <c r="A54" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F54" s="2">
+        <v>2012</v>
+      </c>
+      <c r="G54" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="16">
+      <c r="A55" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B55" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="E55" s="40" t="s">
+        <v>635</v>
+      </c>
+      <c r="F55" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G55" s="19">
+        <v>2028</v>
+      </c>
+      <c r="H55" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="16">
+      <c r="A56" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="B56" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="E56" s="40" t="s">
+        <v>642</v>
+      </c>
+      <c r="F56" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G56" s="19">
+        <v>2031</v>
+      </c>
+      <c r="H56" s="18" t="s">
+        <v>183</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="16">
+      <c r="A57" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="F57" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G57" s="2">
+        <v>2029</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="16">
+      <c r="A58" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="E58" s="24" t="s">
+        <v>191</v>
+      </c>
+      <c r="F58" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G58" s="2">
+        <v>2034</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="16">
+      <c r="A59" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F59" s="2">
+        <v>2013</v>
+      </c>
+      <c r="G59" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="16">
+      <c r="A60" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="F60" s="2">
+        <v>2014</v>
+      </c>
+      <c r="G60" s="2">
+        <v>2037</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="I60" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="16">
+      <c r="A61" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="F61" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G61" s="2">
+        <v>2028</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="16">
+      <c r="A62" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="E62" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="F62" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G62" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I62" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="16">
+      <c r="A63" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="F63" s="2">
+        <v>2018</v>
+      </c>
+      <c r="G63" s="2">
+        <v>2033</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="I63" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="16">
+      <c r="A64" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="F64" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G64" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="16">
+      <c r="A65" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D65" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="E65" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="F65" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G65" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="16">
+      <c r="A66" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="E66" s="40" t="s">
+        <v>643</v>
+      </c>
+      <c r="F66" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G66" s="2">
+        <v>2030</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="16">
+      <c r="A67" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="F67" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G67" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="16">
+      <c r="A68" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="E68" s="24" t="s">
+        <v>234</v>
+      </c>
+      <c r="F68" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G68" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="16">
+      <c r="A69" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="E69" s="45" t="s">
+        <v>238</v>
+      </c>
+      <c r="F69" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G69" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="16">
+      <c r="A70" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="E70" s="24" t="s">
+        <v>242</v>
+      </c>
+      <c r="F70" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G70" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="16">
+      <c r="A71" s="17" t="s">
+        <v>243</v>
+      </c>
+      <c r="B71" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="C71" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D71" s="42" t="s">
+        <v>611</v>
+      </c>
+      <c r="E71" s="42" t="s">
+        <v>612</v>
+      </c>
+      <c r="F71" s="19">
+        <v>2014</v>
+      </c>
+      <c r="G71" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H71" s="18" t="s">
+        <v>245</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="16">
+      <c r="A72" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="B72" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="C72" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D72" s="42" t="s">
+        <v>613</v>
+      </c>
+      <c r="E72" s="47" t="s">
+        <v>636</v>
+      </c>
+      <c r="F72" s="19">
+        <v>2023</v>
+      </c>
+      <c r="G72" s="19">
+        <v>2040</v>
+      </c>
+      <c r="H72" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="16">
+      <c r="A73" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="F73" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G73" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I73" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="16">
+      <c r="A74" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="E74" s="45" t="s">
+        <v>256</v>
+      </c>
+      <c r="F74" s="2">
+        <v>2014</v>
+      </c>
+      <c r="G74" s="2">
+        <v>2029</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="16">
+      <c r="A75" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="B75" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="C75" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D75" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="E75" s="42" t="s">
+        <v>615</v>
+      </c>
+      <c r="F75" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G75" s="19">
+        <v>2039</v>
+      </c>
+      <c r="H75" s="18" t="s">
+        <v>259</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="16">
+      <c r="A76" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="E76" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="F76" s="2">
+        <v>2012</v>
+      </c>
+      <c r="G76" s="2">
+        <v>2029</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="16">
+      <c r="A77" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="F77" s="2">
+        <v>2001</v>
+      </c>
+      <c r="G77" s="2">
+        <v>2021</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="16">
+      <c r="A78" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D78" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="E78" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="F78" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G78" s="2">
+        <v>2036</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="16">
+      <c r="A79" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D79" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="E79" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="F79" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G79" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="16">
+      <c r="A80" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="E80" s="45" t="s">
+        <v>279</v>
+      </c>
+      <c r="F80" s="2">
+        <v>2021</v>
+      </c>
+      <c r="G80" s="2">
+        <v>2039</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="16">
+      <c r="A81" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="B81" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="C81" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D81" s="42" t="s">
+        <v>616</v>
+      </c>
+      <c r="E81" s="47" t="s">
+        <v>637</v>
+      </c>
+      <c r="F81" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G81" s="19">
+        <v>2031</v>
+      </c>
+      <c r="H81" s="18" t="s">
+        <v>282</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="16">
+      <c r="A82" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="B82" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="C82" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D82" s="42" t="s">
+        <v>617</v>
+      </c>
+      <c r="E82" s="47" t="s">
+        <v>638</v>
+      </c>
+      <c r="F82" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G82" s="19">
+        <v>2031</v>
+      </c>
+      <c r="H82" s="18" t="s">
+        <v>285</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="16">
+      <c r="A83" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="B83" s="17" t="s">
+        <v>287</v>
+      </c>
+      <c r="C83" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D83" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="E83" s="42" t="s">
+        <v>615</v>
+      </c>
+      <c r="F83" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G83" s="19">
+        <v>2039</v>
+      </c>
+      <c r="H83" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="16">
+      <c r="A84" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>291</v>
+      </c>
+      <c r="E84" s="45" t="s">
+        <v>292</v>
+      </c>
+      <c r="F84" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G84" s="2">
+        <v>2030</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="16">
+      <c r="A85" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D85" s="45" t="s">
+        <v>295</v>
+      </c>
+      <c r="E85" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="F85" s="2">
+        <v>2010</v>
+      </c>
+      <c r="G85" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I85" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="16">
+      <c r="A86" s="17" t="s">
+        <v>297</v>
+      </c>
+      <c r="B86" s="17" t="s">
+        <v>298</v>
+      </c>
+      <c r="C86" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D86" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="E86" s="42" t="s">
+        <v>615</v>
+      </c>
+      <c r="F86" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G86" s="19">
+        <v>2039</v>
+      </c>
+      <c r="H86" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="16">
+      <c r="A87" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="E87" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="F87" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G87" s="2">
+        <v>2030</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="16">
+      <c r="A88" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="E88" s="45" t="s">
+        <v>307</v>
+      </c>
+      <c r="F88" s="2">
+        <v>2012</v>
+      </c>
+      <c r="G88" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="16">
+      <c r="A89" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="B89" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="C89" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="D89" s="42" t="s">
+        <v>310</v>
+      </c>
+      <c r="E89" s="42" t="s">
+        <v>311</v>
+      </c>
+      <c r="F89" s="19">
+        <v>2008</v>
+      </c>
+      <c r="G89" s="19">
+        <v>2028</v>
+      </c>
+      <c r="H89" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="16">
+      <c r="A90" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D90" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="E90" s="9" t="s">
+        <v>316</v>
+      </c>
+      <c r="F90" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G90" s="2">
+        <v>2025</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="16">
+      <c r="A91" s="17" t="s">
+        <v>317</v>
+      </c>
+      <c r="B91" s="17" t="s">
+        <v>318</v>
+      </c>
+      <c r="C91" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D91" s="42" t="s">
+        <v>618</v>
+      </c>
+      <c r="E91" s="47" t="s">
+        <v>644</v>
+      </c>
+      <c r="F91" s="19">
+        <v>1994</v>
+      </c>
+      <c r="G91" s="19">
+        <v>2025</v>
+      </c>
+      <c r="H91" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="I91" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="16">
+      <c r="A92" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="B92" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="C92" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D92" s="42" t="s">
+        <v>619</v>
+      </c>
+      <c r="E92" s="42" t="s">
+        <v>620</v>
+      </c>
+      <c r="F92" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G92" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H92" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="I92" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="16">
+      <c r="A93" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="C93" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D93" s="9" t="s">
+        <v>325</v>
+      </c>
+      <c r="E93" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="F93" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G93" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I93" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="16">
+      <c r="A94" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D94" s="9" t="s">
+        <v>329</v>
+      </c>
+      <c r="E94" s="45" t="s">
+        <v>330</v>
+      </c>
+      <c r="F94" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G94" s="2">
+        <v>2028</v>
+      </c>
+      <c r="I94" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="16">
+      <c r="A95" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D95" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="E95" s="45" t="s">
+        <v>334</v>
+      </c>
+      <c r="F95" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G95" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I95" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="16">
+      <c r="A96" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D96" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="E96" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="F96" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G96" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I96" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="16">
+      <c r="A97" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C97" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D97" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="E97" s="9" t="s">
+        <v>342</v>
+      </c>
+      <c r="F97" s="2">
+        <v>2004</v>
+      </c>
+      <c r="G97" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="16">
+      <c r="A98" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E98" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="F98" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G98" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" ht="16">
+      <c r="A99" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D99" s="9" t="s">
+        <v>349</v>
+      </c>
+      <c r="E99" s="9" t="s">
+        <v>350</v>
+      </c>
+      <c r="F99" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G99" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" ht="16">
+      <c r="A100" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="B100" s="17" t="s">
+        <v>352</v>
+      </c>
+      <c r="C100" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D100" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="E100" s="42" t="s">
+        <v>615</v>
+      </c>
+      <c r="F100" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G100" s="19">
+        <v>2039</v>
+      </c>
+      <c r="H100" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" ht="16">
+      <c r="A101" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D101" s="9" t="s">
+        <v>356</v>
+      </c>
+      <c r="E101" s="45" t="s">
+        <v>357</v>
+      </c>
+      <c r="F101" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G101" s="2">
+        <v>2033</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" ht="16">
+      <c r="A102" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D102" s="9" t="s">
+        <v>360</v>
+      </c>
+      <c r="E102" s="9" t="s">
+        <v>361</v>
+      </c>
+      <c r="F102" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G102" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" ht="16">
+      <c r="A103" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D103" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="E103" s="45" t="s">
+        <v>365</v>
+      </c>
+      <c r="F103" s="2">
+        <v>2004</v>
+      </c>
+      <c r="G103" s="2">
+        <v>2021</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" ht="16">
+      <c r="A104" s="27" t="s">
+        <v>366</v>
+      </c>
+      <c r="B104" s="27" t="s">
+        <v>367</v>
+      </c>
+      <c r="C104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="G104" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="H104" s="29" t="s">
+        <v>368</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" ht="16">
+      <c r="A105" s="15" t="s">
+        <v>673</v>
+      </c>
+      <c r="B105" s="15" t="s">
+        <v>674</v>
+      </c>
+      <c r="C105" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D105" s="41" t="s">
+        <v>369</v>
+      </c>
+      <c r="E105" s="41" t="s">
+        <v>370</v>
+      </c>
+      <c r="F105" s="16">
+        <v>2006</v>
+      </c>
+      <c r="G105" s="16">
+        <v>2029</v>
+      </c>
+      <c r="H105" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" ht="16">
+      <c r="A106" s="15" t="s">
+        <v>675</v>
+      </c>
+      <c r="B106" s="15" t="s">
+        <v>676</v>
+      </c>
+      <c r="C106" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D106" s="41" t="s">
+        <v>372</v>
+      </c>
+      <c r="E106" s="41" t="s">
+        <v>373</v>
+      </c>
+      <c r="F106" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G106" s="16">
+        <v>2032</v>
+      </c>
+      <c r="H106" s="10" t="s">
+        <v>374</v>
+      </c>
+      <c r="I106" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" ht="16">
+      <c r="A107" s="15" t="s">
+        <v>677</v>
+      </c>
+      <c r="B107" s="15" t="s">
+        <v>678</v>
+      </c>
+      <c r="C107" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D107" s="41" t="s">
+        <v>375</v>
+      </c>
+      <c r="E107" s="41" t="s">
+        <v>376</v>
+      </c>
+      <c r="F107" s="16">
+        <v>2012</v>
+      </c>
+      <c r="G107" s="16">
+        <v>2032</v>
+      </c>
+      <c r="H107" s="10" t="s">
+        <v>377</v>
+      </c>
+      <c r="I107" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" ht="16">
+      <c r="A108" s="15" t="s">
+        <v>679</v>
+      </c>
+      <c r="B108" s="15" t="s">
+        <v>680</v>
+      </c>
+      <c r="C108" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D108" s="41" t="s">
+        <v>375</v>
+      </c>
+      <c r="E108" s="41" t="s">
+        <v>378</v>
+      </c>
+      <c r="F108" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G108" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H108" s="10" t="s">
+        <v>379</v>
+      </c>
+      <c r="I108" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" ht="16">
+      <c r="A109" s="15" t="s">
+        <v>681</v>
+      </c>
+      <c r="B109" s="15" t="s">
+        <v>682</v>
+      </c>
+      <c r="C109" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D109" s="41" t="s">
+        <v>380</v>
+      </c>
+      <c r="E109" s="41" t="s">
+        <v>381</v>
+      </c>
+      <c r="F109" s="16">
+        <v>2006</v>
+      </c>
+      <c r="G109" s="16">
+        <v>2028</v>
+      </c>
+      <c r="H109" s="10" t="s">
+        <v>382</v>
+      </c>
+      <c r="I109" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" ht="16">
+      <c r="A110" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D110" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="E110" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="F110" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G110" s="2">
+        <v>2028</v>
+      </c>
+      <c r="I110" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" ht="16">
+      <c r="A111" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D111" s="9" t="s">
+        <v>389</v>
+      </c>
+      <c r="E111" s="9" t="s">
+        <v>390</v>
+      </c>
+      <c r="F111" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G111" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I111" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" ht="16">
+      <c r="A112" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D112" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="E112" s="9" t="s">
+        <v>394</v>
+      </c>
+      <c r="F112" s="2">
+        <v>2013</v>
+      </c>
+      <c r="G112" s="2">
+        <v>2033</v>
+      </c>
+      <c r="I112" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" ht="16">
+      <c r="A113" s="17" t="s">
+        <v>395</v>
+      </c>
+      <c r="B113" s="17" t="s">
+        <v>396</v>
+      </c>
+      <c r="C113" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D113" s="42" t="s">
+        <v>621</v>
+      </c>
+      <c r="E113" s="42" t="s">
+        <v>622</v>
+      </c>
+      <c r="F113" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G113" s="19">
+        <v>2031</v>
+      </c>
+      <c r="H113" s="18" t="s">
+        <v>397</v>
+      </c>
+      <c r="I113" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" ht="16">
+      <c r="A114" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D114" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="E114" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="F114" s="2">
+        <v>2001</v>
+      </c>
+      <c r="G114" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I114" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" ht="16">
+      <c r="A115" s="17" t="s">
+        <v>402</v>
+      </c>
+      <c r="B115" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="C115" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D115" s="42" t="s">
+        <v>614</v>
+      </c>
+      <c r="E115" s="42" t="s">
+        <v>615</v>
+      </c>
+      <c r="F115" s="19">
+        <v>2022</v>
+      </c>
+      <c r="G115" s="19">
+        <v>2039</v>
+      </c>
+      <c r="H115" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="I115" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" ht="16">
+      <c r="A116" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D116" s="9" t="s">
+        <v>407</v>
+      </c>
+      <c r="E116" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="F116" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G116" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I116" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" ht="16">
+      <c r="A117" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="C117" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D117" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="E117" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="F117" s="2">
+        <v>2013</v>
+      </c>
+      <c r="G117" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I117" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" ht="16">
+      <c r="A118" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="C118" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D118" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="E118" s="9" t="s">
+        <v>416</v>
+      </c>
+      <c r="F118" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G118" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I118" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" ht="16">
+      <c r="A119" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C119" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D119" s="9" t="s">
+        <v>419</v>
+      </c>
+      <c r="E119" s="24" t="s">
+        <v>420</v>
+      </c>
+      <c r="F119" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G119" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I119" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" ht="16">
+      <c r="A120" s="17" t="s">
+        <v>421</v>
+      </c>
+      <c r="B120" s="17" t="s">
+        <v>422</v>
+      </c>
+      <c r="C120" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D120" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="E120" s="40" t="s">
+        <v>639</v>
+      </c>
+      <c r="F120" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G120" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H120" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="I120" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" ht="16">
+      <c r="A121" s="17" t="s">
+        <v>424</v>
+      </c>
+      <c r="B121" s="17" t="s">
+        <v>425</v>
+      </c>
+      <c r="C121" s="19" t="s">
+        <v>27</v>
+      </c>
+      <c r="D121" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="E121" s="40" t="s">
+        <v>639</v>
+      </c>
+      <c r="F121" s="19">
+        <v>2011</v>
+      </c>
+      <c r="G121" s="19">
+        <v>2026</v>
+      </c>
+      <c r="H121" s="18" t="s">
+        <v>426</v>
+      </c>
+      <c r="I121" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" ht="16">
+      <c r="A122" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="C122" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D122" s="9" t="s">
+        <v>429</v>
+      </c>
+      <c r="E122" s="9" t="s">
+        <v>430</v>
+      </c>
+      <c r="F122" s="2">
+        <v>2023</v>
+      </c>
+      <c r="G122" s="2">
+        <v>2038</v>
+      </c>
+      <c r="I122" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" ht="16">
+      <c r="A123" s="27" t="s">
+        <v>431</v>
+      </c>
+      <c r="B123" s="27" t="s">
+        <v>432</v>
+      </c>
+      <c r="C123" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="D123" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E123" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="G123" s="28" t="s">
+        <v>11</v>
+      </c>
+      <c r="H123" s="29" t="s">
+        <v>433</v>
+      </c>
+      <c r="I123" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" ht="16">
+      <c r="A124" s="16" t="s">
+        <v>683</v>
+      </c>
+      <c r="B124" s="16" t="s">
+        <v>684</v>
+      </c>
+      <c r="C124" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D124" s="41" t="s">
+        <v>434</v>
+      </c>
+      <c r="E124" s="41" t="s">
+        <v>435</v>
+      </c>
+      <c r="F124" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G124" s="16">
+        <v>2029</v>
+      </c>
+      <c r="H124" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="I124" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" ht="16">
+      <c r="A125" s="16" t="s">
+        <v>685</v>
+      </c>
+      <c r="B125" s="16" t="s">
+        <v>686</v>
+      </c>
+      <c r="C125" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D125" s="41" t="s">
+        <v>434</v>
+      </c>
+      <c r="E125" s="41" t="s">
+        <v>435</v>
+      </c>
+      <c r="F125" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G125" s="16">
+        <v>2029</v>
+      </c>
+      <c r="H125" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="I125" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" ht="16">
+      <c r="A126" s="16" t="s">
+        <v>687</v>
+      </c>
+      <c r="B126" s="16" t="s">
+        <v>688</v>
+      </c>
+      <c r="C126" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D126" s="41" t="s">
+        <v>434</v>
+      </c>
+      <c r="E126" s="41" t="s">
+        <v>435</v>
+      </c>
+      <c r="F126" s="16">
+        <v>2011</v>
+      </c>
+      <c r="G126" s="16">
+        <v>2029</v>
+      </c>
+      <c r="H126" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="I126" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" ht="16">
+      <c r="A127" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C127" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D127" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="E127" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="F127" s="2">
+        <v>2010</v>
+      </c>
+      <c r="G127" s="2">
+        <v>2027</v>
+      </c>
+      <c r="I127" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" ht="16">
+      <c r="A128" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C128" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D128" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="E128" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="F128" s="2">
+        <v>2006</v>
+      </c>
+      <c r="G128" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I128" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" ht="16">
+      <c r="A129" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C129" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D129" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E129" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="F129" s="2">
+        <v>2023</v>
+      </c>
+      <c r="G129" s="2">
+        <v>2040</v>
+      </c>
+      <c r="H129" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="I129" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" ht="16">
+      <c r="A130" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C130" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D130" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="E130" s="24" t="s">
+        <v>453</v>
+      </c>
+      <c r="F130" s="2">
+        <v>2024</v>
+      </c>
+      <c r="G130" s="2">
+        <v>2041</v>
+      </c>
+      <c r="I130" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" ht="16">
+      <c r="A131" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="C131" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D131" s="9" t="s">
+        <v>456</v>
+      </c>
+      <c r="E131" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="F131" s="2">
+        <v>2020</v>
+      </c>
+      <c r="G131" s="2">
+        <v>2035</v>
+      </c>
+      <c r="I131" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" ht="16">
+      <c r="A132" s="30" t="s">
+        <v>458</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="C132" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D132" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="E132" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="F132" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G132" s="2">
+        <v>2030</v>
+      </c>
+      <c r="I132" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" ht="16">
+      <c r="A133" s="30" t="s">
+        <v>462</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C133" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D133" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="E133" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="F133" s="2">
+        <v>2015</v>
+      </c>
+      <c r="G133" s="2">
+        <v>2036</v>
+      </c>
+      <c r="I133" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" ht="16">
+      <c r="A134" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="C134" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D134" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="E134" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="F134" s="2">
+        <v>2016</v>
+      </c>
+      <c r="G134" s="2">
+        <v>2035</v>
+      </c>
+      <c r="I134" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" ht="16">
+      <c r="A135" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C135" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D135" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="E135" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="F135" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G135" s="2">
+        <v>2031</v>
+      </c>
+      <c r="I135" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" ht="16">
+      <c r="A136" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B136" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C136" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D136" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="E136" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="F136" s="2">
+        <v>2017</v>
+      </c>
+      <c r="G136" s="2">
+        <v>2037</v>
+      </c>
+      <c r="I136" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" ht="16">
+      <c r="A137" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B137" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="C137" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D137" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="E137" s="45" t="s">
+        <v>481</v>
+      </c>
+      <c r="F137" s="2">
+        <v>2011</v>
+      </c>
+      <c r="G137" s="2">
+        <v>2026</v>
+      </c>
+      <c r="I137" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D27" r:id="rId1" xr:uid="{92578C69-2E4F-C741-AF5B-DA2D9BC42273}"/>
+    <hyperlink ref="E27" r:id="rId2" xr:uid="{173F19DC-D9E0-DE40-BAC5-C505F83D50A3}"/>
+    <hyperlink ref="D28" r:id="rId3" xr:uid="{D1665A1B-11A8-614C-B25D-F495A8767CE8}"/>
+    <hyperlink ref="E28" r:id="rId4" xr:uid="{684C7EAB-4A30-704E-B5EA-87ADD38EE503}"/>
+    <hyperlink ref="D29" r:id="rId5" xr:uid="{1517C533-7019-F846-A298-9E1F9A8EF414}"/>
+    <hyperlink ref="E29" r:id="rId6" xr:uid="{DCD6095C-1DFB-2749-AD13-27F27E1BAA31}"/>
+    <hyperlink ref="D30" r:id="rId7" xr:uid="{DB34845A-30BF-D143-A19C-04895E655106}"/>
+    <hyperlink ref="D31" r:id="rId8" xr:uid="{FE0AB7F8-B531-A949-92B6-E18CF272F31B}"/>
+    <hyperlink ref="E31" r:id="rId9" xr:uid="{80A5A031-F54D-DB4E-A01C-84D47A8240EF}"/>
+    <hyperlink ref="D32" r:id="rId10" xr:uid="{FC118876-3653-B544-A557-862FFE1AFC02}"/>
+    <hyperlink ref="E32" r:id="rId11" xr:uid="{EEE9AD74-BABF-724F-AA58-9832A98F3272}"/>
+    <hyperlink ref="D33" r:id="rId12" location="page-1" xr:uid="{8ED80BEE-ACAA-9946-B9C6-6D1BF2F77B17}"/>
+    <hyperlink ref="E33" r:id="rId13" xr:uid="{D5F76272-B5E5-A74C-BD31-05957955B581}"/>
+    <hyperlink ref="E41" r:id="rId14" xr:uid="{D0B23B98-4224-0149-9B46-97CAC7CBB109}"/>
+    <hyperlink ref="D42" r:id="rId15" xr:uid="{1D8A72A8-DAAD-FE40-8E0E-7519EACFCACE}"/>
+    <hyperlink ref="E42" r:id="rId16" xr:uid="{08088A6A-03C5-8741-9EE7-52CAD760A8D3}"/>
+    <hyperlink ref="D43" r:id="rId17" xr:uid="{CB2C19CB-3CB6-524A-A594-CA6DC0627DF1}"/>
+    <hyperlink ref="E43" r:id="rId18" xr:uid="{B7717258-84AB-8E41-AE3F-31B744E11350}"/>
+    <hyperlink ref="D44" r:id="rId19" xr:uid="{6CB9E2EF-5993-854C-904E-00754740D903}"/>
+    <hyperlink ref="E44" r:id="rId20" xr:uid="{E3581571-A360-994A-80F2-4D4A87D0D724}"/>
+    <hyperlink ref="H44" r:id="rId21" xr:uid="{483FF2C9-F84A-6843-B611-E331143EB1E4}"/>
+    <hyperlink ref="D45" r:id="rId22" xr:uid="{A20097A4-2350-3049-ACB6-5DA283D33190}"/>
+    <hyperlink ref="E45" r:id="rId23" xr:uid="{837D2D69-D1B4-C94B-9BC1-6815C046AF70}"/>
+    <hyperlink ref="D46" r:id="rId24" xr:uid="{3900B938-16C6-4D4C-8E70-D90896EA5F34}"/>
+    <hyperlink ref="E46" r:id="rId25" xr:uid="{B00B71C5-D0CE-C841-BDCF-7DF2A1E295C2}"/>
+    <hyperlink ref="D47" r:id="rId26" location="core-strategy-2010" xr:uid="{0A40E3A6-BE98-F549-8FD2-9B2B3926CD24}"/>
+    <hyperlink ref="E47" r:id="rId27" xr:uid="{528A4500-DEF0-FC46-94DD-197756397FA2}"/>
+    <hyperlink ref="D48" r:id="rId28" xr:uid="{5DE2EA7A-DA82-5B4B-A079-CCCE8E9FFC24}"/>
+    <hyperlink ref="E48" r:id="rId29" xr:uid="{8100A349-FF07-934E-A695-12E6B75CC2CE}"/>
+    <hyperlink ref="D50" r:id="rId30" xr:uid="{B5186A23-984D-244A-BB49-FDB34EE80B49}"/>
+    <hyperlink ref="E50" r:id="rId31" xr:uid="{99408002-64BD-E547-9773-6E1907A5C720}"/>
+    <hyperlink ref="D54" r:id="rId32" xr:uid="{7F57EDE3-01D0-0445-99BE-510E06E7F7E0}"/>
+    <hyperlink ref="E54" r:id="rId33" xr:uid="{EC9A62D3-0F8C-674D-8F1D-87C1E1EB3836}"/>
+    <hyperlink ref="D55" r:id="rId34" xr:uid="{5343CAAC-BF3B-FE48-B71A-F4834D1EB9D3}"/>
+    <hyperlink ref="E56" r:id="rId35" xr:uid="{F176CBAC-932F-E247-B7BC-BA16AF9CF925}"/>
+    <hyperlink ref="D57" r:id="rId36" xr:uid="{74CDF1CE-732F-3C4F-8B7F-4AB9DE257E46}"/>
+    <hyperlink ref="E57" r:id="rId37" xr:uid="{1D551FFD-17C0-E54E-954C-851B8153878D}"/>
+    <hyperlink ref="D58" r:id="rId38" xr:uid="{613B96D7-9F18-D142-B289-2B8E30A09BEF}"/>
+    <hyperlink ref="E58" r:id="rId39" xr:uid="{9CB5F426-3702-BC4A-BE6D-2E652BA07266}"/>
+    <hyperlink ref="D59" r:id="rId40" xr:uid="{BBCFDC87-1822-F949-BF31-0A6BC4D91150}"/>
+    <hyperlink ref="E59" r:id="rId41" xr:uid="{55BF4782-7D00-8844-A91E-240A6C1BE2D3}"/>
+    <hyperlink ref="D60" r:id="rId42" xr:uid="{15D2D70B-A288-FE44-845F-F18BEE868CA3}"/>
+    <hyperlink ref="E60" r:id="rId43" xr:uid="{C052A175-EA4B-A54F-B0C4-45C27D149811}"/>
+    <hyperlink ref="D61" r:id="rId44" xr:uid="{ED41D30D-F331-9247-A9E4-FC4146FCC5F8}"/>
+    <hyperlink ref="E61" r:id="rId45" xr:uid="{13FD7C79-DCEA-CE4E-96FF-175DC0F5C4B2}"/>
+    <hyperlink ref="D62" r:id="rId46" xr:uid="{CC8C8521-6E9F-DC4C-8D19-C45EE989DCBA}"/>
+    <hyperlink ref="E62" r:id="rId47" xr:uid="{251854FC-CCAF-F24D-87F7-A381ABEC986C}"/>
+    <hyperlink ref="D63" r:id="rId48" xr:uid="{B73E719B-1DAC-F049-B51B-BA5DCBCF2820}"/>
+    <hyperlink ref="E63" r:id="rId49" xr:uid="{0FCE6EFA-B1E4-6149-994E-8B8E5D675D26}"/>
+    <hyperlink ref="D64" r:id="rId50" xr:uid="{EB491F76-D318-3648-AE5B-4C5F70AFB2DF}"/>
+    <hyperlink ref="E64" r:id="rId51" xr:uid="{9FD3352C-1268-6546-BD0E-455DB358B6B5}"/>
+    <hyperlink ref="D65" r:id="rId52" xr:uid="{6014FD44-BE28-7144-9925-650C3667281D}"/>
+    <hyperlink ref="E65" r:id="rId53" xr:uid="{1F95395F-08A1-6740-8A2E-E80A66B98048}"/>
+    <hyperlink ref="D66" r:id="rId54" xr:uid="{28B560E0-D64B-0747-9417-2A88195F124B}"/>
+    <hyperlink ref="E66" r:id="rId55" xr:uid="{EEDEA802-F6A2-1F4B-B872-A210C1A26376}"/>
+    <hyperlink ref="D67" r:id="rId56" xr:uid="{FAA8F0EF-9BFC-9846-99D0-0A0B0C902FC7}"/>
+    <hyperlink ref="E67" r:id="rId57" xr:uid="{68927A1D-6059-F944-9B9F-4E11813E0563}"/>
+    <hyperlink ref="D68" r:id="rId58" xr:uid="{B8764A21-DFA4-4F44-A050-5754ABAD6A2E}"/>
+    <hyperlink ref="E68" r:id="rId59" xr:uid="{1CF28895-DCE7-B848-99ED-1EBA8BB1EFBD}"/>
+    <hyperlink ref="D69" r:id="rId60" xr:uid="{B0A52BF6-6DA7-644A-A9CF-7535E559493F}"/>
+    <hyperlink ref="E69" r:id="rId61" xr:uid="{74FB13FF-AC6D-F446-B627-7DB34159544C}"/>
+    <hyperlink ref="D70" r:id="rId62" xr:uid="{181832B5-A85B-A54E-8C62-3BE0861A2F5C}"/>
+    <hyperlink ref="E70" r:id="rId63" xr:uid="{05CFBA40-A7C0-BF40-9A2E-7A2BECE3C002}"/>
+    <hyperlink ref="D73" r:id="rId64" xr:uid="{9AEA6F4D-B221-764C-868C-1B2D37890C15}"/>
+    <hyperlink ref="E73" r:id="rId65" xr:uid="{D2D48D4F-BFDA-FB4B-86A7-66DD1E7B6267}"/>
+    <hyperlink ref="D74" r:id="rId66" xr:uid="{99DC8D53-0B89-334C-8773-4B2CB271737F}"/>
+    <hyperlink ref="E74" r:id="rId67" xr:uid="{FA592C8E-A54E-0144-BDB3-5751164DD3F4}"/>
+    <hyperlink ref="D76" r:id="rId68" xr:uid="{78CFED17-1757-0F42-BBE0-F4A8B3317D44}"/>
+    <hyperlink ref="E76" r:id="rId69" xr:uid="{EA32C56C-C451-0E44-909C-1C531B249325}"/>
+    <hyperlink ref="D77" r:id="rId70" xr:uid="{D00294DF-FF62-1A49-85AF-F40DDE9F2926}"/>
+    <hyperlink ref="E77" r:id="rId71" xr:uid="{0E879C1D-0351-2A49-95B5-68AAC3017143}"/>
+    <hyperlink ref="D78" r:id="rId72" xr:uid="{4A553D58-B6AA-FF49-A5D5-ABEF3C574392}"/>
+    <hyperlink ref="E78" r:id="rId73" xr:uid="{AE4A40FD-5A22-D34F-8CA7-BF6C2F9CC703}"/>
+    <hyperlink ref="D79" r:id="rId74" xr:uid="{EA05C89E-CC04-9741-91F7-5D485C616EEE}"/>
+    <hyperlink ref="E79" r:id="rId75" xr:uid="{2D8F9EEB-B4C9-5647-97AE-26A1D8A95C1D}"/>
+    <hyperlink ref="D80" r:id="rId76" xr:uid="{37467B4D-D6FA-2B46-9482-10F0329668D5}"/>
+    <hyperlink ref="E80" r:id="rId77" xr:uid="{4AC6B72E-6F4C-9940-B9CA-01A5FC28D3EE}"/>
+    <hyperlink ref="D84" r:id="rId78" xr:uid="{3FBD1905-CF6F-D94C-A143-947A93F60C4C}"/>
+    <hyperlink ref="E84" r:id="rId79" xr:uid="{2A58ADFC-0EAC-2C46-86AA-A301A9E38DD7}"/>
+    <hyperlink ref="D85" r:id="rId80" xr:uid="{CB2C61BA-21E2-B846-AAFE-5F51F9592976}"/>
+    <hyperlink ref="E85" r:id="rId81" xr:uid="{FB467818-E823-AB4E-8019-C12A55E9CAFF}"/>
+    <hyperlink ref="D87" r:id="rId82" xr:uid="{63A33E0D-24DB-8345-8663-1A678A1779F4}"/>
+    <hyperlink ref="E87" r:id="rId83" xr:uid="{D962CCCC-4761-4E47-A856-91A08F287C27}"/>
+    <hyperlink ref="D88" r:id="rId84" xr:uid="{3E3043FC-174E-2A43-BA3F-F0DE496A8003}"/>
+    <hyperlink ref="E88" r:id="rId85" xr:uid="{0FDCC4EF-13D4-E046-A161-43CD4C083F43}"/>
+    <hyperlink ref="D89" r:id="rId86" xr:uid="{8BE9D0E6-A1FB-AF43-AC0E-9E4743243FCB}"/>
+    <hyperlink ref="E89" r:id="rId87" xr:uid="{740A9239-FA53-1743-91E9-ED734183D2C7}"/>
+    <hyperlink ref="D90" r:id="rId88" xr:uid="{6863BE1D-E69D-FC49-91EE-84FF3B3FF246}"/>
+    <hyperlink ref="E90" r:id="rId89" xr:uid="{AECDB259-8F76-5549-8117-E929184AF844}"/>
+    <hyperlink ref="D93" r:id="rId90" xr:uid="{653AFE77-5E3E-974A-A801-96499F32BE92}"/>
+    <hyperlink ref="E93" r:id="rId91" xr:uid="{6EF6C82F-3205-574D-A5D2-8DE37EF0D7F7}"/>
+    <hyperlink ref="D94" r:id="rId92" xr:uid="{13E099F3-1C2E-8045-9104-9ECF975123E4}"/>
+    <hyperlink ref="E94" r:id="rId93" xr:uid="{615F7038-8B00-7046-A4C8-DA76551FD4B7}"/>
+    <hyperlink ref="D95" r:id="rId94" xr:uid="{84CFCF8D-ECC6-364B-B181-92A0E796A8FB}"/>
+    <hyperlink ref="E95" r:id="rId95" xr:uid="{1D91EA12-959A-9248-974D-5A8B4BB762DF}"/>
+    <hyperlink ref="D96" r:id="rId96" xr:uid="{21B3F400-01FF-6441-808D-DCDD3189A75D}"/>
+    <hyperlink ref="E96" r:id="rId97" xr:uid="{FB472213-15DD-E042-AF07-F72333B66ED6}"/>
+    <hyperlink ref="D97" r:id="rId98" xr:uid="{5FC50E96-EEB8-2343-B2F7-4FDDFB9222DB}"/>
+    <hyperlink ref="E97" r:id="rId99" xr:uid="{7472185E-F447-F44E-9ECB-397C543E0A1C}"/>
+    <hyperlink ref="D98" r:id="rId100" xr:uid="{4C15C43E-13A0-134A-B161-5A302BDCB76C}"/>
+    <hyperlink ref="E98" r:id="rId101" xr:uid="{08F89DB9-2E71-274E-BB4C-9805BEEC8969}"/>
+    <hyperlink ref="D99" r:id="rId102" xr:uid="{24723E9B-E1F1-D449-95BC-AC4E4A1F16C4}"/>
+    <hyperlink ref="E99" r:id="rId103" xr:uid="{FE62D18C-7A10-834B-A327-9FA58182C9A5}"/>
+    <hyperlink ref="D101" r:id="rId104" xr:uid="{CBE8F476-FF7F-E541-BA54-B3EA8E6FE201}"/>
+    <hyperlink ref="E101" r:id="rId105" xr:uid="{D4CFF67C-E453-C040-ABF1-B65D6055768B}"/>
+    <hyperlink ref="D102" r:id="rId106" xr:uid="{CEE8A011-E81C-5D4D-B22A-364F7C52A653}"/>
+    <hyperlink ref="E102" r:id="rId107" xr:uid="{8E0B5897-C9E3-F04B-853B-544838E8D7F6}"/>
+    <hyperlink ref="D103" r:id="rId108" xr:uid="{A50E66E4-A856-544B-BD69-5D992DF5D2EF}"/>
+    <hyperlink ref="E103" r:id="rId109" xr:uid="{9B2B86DD-A8EE-924D-A9B6-78CA4CA7DD8E}"/>
+    <hyperlink ref="D110" r:id="rId110" xr:uid="{9009F9AD-5E70-724D-B81F-9F2302F20402}"/>
+    <hyperlink ref="E110" r:id="rId111" xr:uid="{A7CD1D0C-D47B-FA45-A186-B1D034E0C4C6}"/>
+    <hyperlink ref="D111" r:id="rId112" xr:uid="{08BCAA3B-8D82-C442-87EF-8A4318C1AADF}"/>
+    <hyperlink ref="E111" r:id="rId113" xr:uid="{9A7A1E1D-8945-9447-B3F6-F2CAB548E858}"/>
+    <hyperlink ref="D112" r:id="rId114" xr:uid="{1E6E8758-55A5-C740-884D-1288EDF679F4}"/>
+    <hyperlink ref="E112" r:id="rId115" xr:uid="{D196471B-37FC-5B48-8FE3-8ADD83FCACE7}"/>
+    <hyperlink ref="D114" r:id="rId116" xr:uid="{BF088E58-BF46-E74E-BBB6-1A89DF9246B8}"/>
+    <hyperlink ref="E114" r:id="rId117" xr:uid="{7102A4FC-04ED-0248-8CFA-F8CDE78A2820}"/>
+    <hyperlink ref="D116" r:id="rId118" xr:uid="{5196DD57-FA51-B54E-B07D-44FEC1ACEFB8}"/>
+    <hyperlink ref="E116" r:id="rId119" xr:uid="{0F5EBA4A-34FA-B246-9B1D-3F2CFAB51255}"/>
+    <hyperlink ref="D117" r:id="rId120" xr:uid="{17126AE6-AAC8-2B4E-A684-61032C18BFF3}"/>
+    <hyperlink ref="E117" r:id="rId121" xr:uid="{88D0E8F8-BAA3-724D-AB8D-3BD6D68A12A1}"/>
+    <hyperlink ref="D118" r:id="rId122" xr:uid="{7BD9258B-70FB-C046-A2FE-CCC96F041FB5}"/>
+    <hyperlink ref="E118" r:id="rId123" xr:uid="{52BF479F-FF2B-A342-9909-905A958BF33E}"/>
+    <hyperlink ref="D119" r:id="rId124" xr:uid="{9A5C9D3E-174C-A544-B79F-61848A2C4C32}"/>
+    <hyperlink ref="E119" r:id="rId125" xr:uid="{28EB3875-403C-044A-8525-E4E059C44C4F}"/>
+    <hyperlink ref="D122" r:id="rId126" xr:uid="{A6AB18E6-5576-C447-9792-BBE68EB06B9C}"/>
+    <hyperlink ref="E122" r:id="rId127" xr:uid="{D54D947B-D764-A241-95E2-9F02223AC208}"/>
+    <hyperlink ref="D127" r:id="rId128" xr:uid="{15DEA36C-4467-7142-8FAF-4DBDF2F7F8C9}"/>
+    <hyperlink ref="E127" r:id="rId129" xr:uid="{95378B09-3D5B-9141-88F8-F472ECC5ED40}"/>
+    <hyperlink ref="D128" r:id="rId130" xr:uid="{E8191620-073B-F44C-A68B-B82926B871B3}"/>
+    <hyperlink ref="E128" r:id="rId131" xr:uid="{D3B6B439-365B-8A42-A606-4D1B3291745B}"/>
+    <hyperlink ref="D129" r:id="rId132" xr:uid="{CD69548E-49B5-B949-8E22-2BE4DCFF4487}"/>
+    <hyperlink ref="E129" r:id="rId133" xr:uid="{45A1B1DD-AFF8-E04F-B711-E25AED2F036C}"/>
+    <hyperlink ref="D130" r:id="rId134" xr:uid="{158ACE7B-ED9F-DE46-8F1B-9954753B2D05}"/>
+    <hyperlink ref="E130" r:id="rId135" xr:uid="{5FB617BC-9252-644F-B5FB-A50D61393E57}"/>
+    <hyperlink ref="D131" r:id="rId136" xr:uid="{CC6C8C01-6F71-2B42-BD69-904F1AF07018}"/>
+    <hyperlink ref="E131" r:id="rId137" xr:uid="{3BFF8D07-BBAB-254A-B626-5A1BFB2890DC}"/>
+    <hyperlink ref="D132" r:id="rId138" xr:uid="{1639C071-87C5-AF47-8854-9523A244FB54}"/>
+    <hyperlink ref="E132" r:id="rId139" xr:uid="{84106256-3EDB-D249-A141-3E969D815AFA}"/>
+    <hyperlink ref="D133" r:id="rId140" xr:uid="{DFEBEAD0-DEA6-2A44-B715-9BCAF8DDD86B}"/>
+    <hyperlink ref="E133" r:id="rId141" xr:uid="{97DC37B9-B350-8445-9AB1-CDBC2A84FCF8}"/>
+    <hyperlink ref="D134" r:id="rId142" xr:uid="{1BE0D959-5493-7C47-96DF-B9DA748CC5A0}"/>
+    <hyperlink ref="E134" r:id="rId143" xr:uid="{EB14CBAE-BF21-C845-9BF8-1F0FAD0F2293}"/>
+    <hyperlink ref="D135" r:id="rId144" xr:uid="{24692671-B35C-724B-A0F1-A3A6B40538B7}"/>
+    <hyperlink ref="E135" r:id="rId145" xr:uid="{7D0A4260-2583-AA42-ABEC-9F87A25C4FD5}"/>
+    <hyperlink ref="D136" r:id="rId146" xr:uid="{E06EF4ED-0454-2F4D-BA1C-FBE37A59049D}"/>
+    <hyperlink ref="E136" r:id="rId147" xr:uid="{88BFD99B-580D-B64F-A4D3-88BE04A8590A}"/>
+    <hyperlink ref="D137" r:id="rId148" xr:uid="{AB6D96E1-6E47-184A-B166-2B68DB92BCF3}"/>
+    <hyperlink ref="E137" r:id="rId149" xr:uid="{60CF3DFB-7F82-3941-9145-CF95180F8094}"/>
+    <hyperlink ref="E6" r:id="rId150" xr:uid="{A36BE10C-45CD-E04E-9BD5-48BCB9042176}"/>
+    <hyperlink ref="E5" r:id="rId151" xr:uid="{0DAEF8C5-9741-0744-A324-5F1E35755B00}"/>
+    <hyperlink ref="E13" r:id="rId152" xr:uid="{631BD9DB-DC3C-2B44-8829-D7CF56153267}"/>
+    <hyperlink ref="E23" r:id="rId153" xr:uid="{6442D484-5B7D-F34C-BAC7-976AE9A53FBE}"/>
+    <hyperlink ref="E49" r:id="rId154" xr:uid="{7A9C2E3E-1956-7C4E-A48B-6F6E9F8E3259}"/>
+    <hyperlink ref="E55" r:id="rId155" xr:uid="{1D0956F2-9408-564F-B888-ED0E839130A7}"/>
+    <hyperlink ref="E72" r:id="rId156" xr:uid="{298D256B-8E41-1C46-908D-1BAC885104E5}"/>
+    <hyperlink ref="E81" r:id="rId157" xr:uid="{B6F587D2-A905-7A4E-9E3D-D86B6D85099E}"/>
+    <hyperlink ref="E82" r:id="rId158" xr:uid="{1CC16E95-3540-4A49-A2DD-CF074CC8C248}"/>
+    <hyperlink ref="E120" r:id="rId159" xr:uid="{5704BDFE-7C41-B342-9631-BCC727417F2F}"/>
+    <hyperlink ref="E121" r:id="rId160" xr:uid="{8AE99BFE-ED4A-8247-8C92-0549957F0C23}"/>
+    <hyperlink ref="E22" r:id="rId161" display="https://centralbedfordshirecouncil.sharepoint.com/sites/Communications/Website and intranet/Forms/AllItems.aspx?id=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2FCentral%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035%2Epdf&amp;parent=%2Fsites%2FCommunications%2FWebsite%20and%20intranet%2FWebsite%20Documents%2FPlanning%2FLocal%20Plan%2FLocal%20Plan%20Documents%2F15%5F%20Adoption%20documents%2F2%5F%20Central%20Bedfordshire%20Local%20Plan%202015%20%E2%80%93%202035&amp;p=true&amp;ga=1" xr:uid="{E832FE20-7EB7-394F-A3EC-8268C42AF05A}"/>
+    <hyperlink ref="D22" r:id="rId162" xr:uid="{475B7D51-8852-F04C-9C84-727A8321DBA2}"/>
+    <hyperlink ref="E26" r:id="rId163" xr:uid="{50388661-06E5-C144-86C3-6352DAF1E143}"/>
+    <hyperlink ref="E91" r:id="rId164" xr:uid="{38B537D8-AB96-4C4A-BADA-9DEDF84E5D05}"/>
+    <hyperlink ref="D35" r:id="rId165" xr:uid="{3A7AC69C-0FED-D844-952E-87E09BCD5EB2}"/>
+    <hyperlink ref="E35" r:id="rId166" xr:uid="{121AEC3A-FFC5-F441-A06A-21AC2BB05E8E}"/>
+    <hyperlink ref="D36" r:id="rId167" xr:uid="{B82FB4DA-4FB3-D245-8454-49D3C9E91309}"/>
+    <hyperlink ref="E36" r:id="rId168" xr:uid="{2FF16388-054C-9745-940D-45BB74BCA011}"/>
+    <hyperlink ref="D37" r:id="rId169" xr:uid="{3770847D-40CD-554C-843C-D041EDB20E3E}"/>
+    <hyperlink ref="E37" r:id="rId170" xr:uid="{00B77E62-922C-204D-BA63-A0BB56E422D8}"/>
+    <hyperlink ref="D38" r:id="rId171" xr:uid="{2D1DBBBE-417D-364D-974D-E3134EE50330}"/>
+    <hyperlink ref="E38" r:id="rId172" xr:uid="{6AE929A5-9DC8-E746-90C2-9E21281239BF}"/>
+    <hyperlink ref="D40" r:id="rId173" xr:uid="{BCF8FC8A-FC94-EE43-9269-BFD32EF551AC}"/>
+    <hyperlink ref="E40" r:id="rId174" xr:uid="{795BC141-190C-2E4E-9AB6-86E23CB5445E}"/>
+    <hyperlink ref="D39" r:id="rId175" xr:uid="{899D9F54-2943-5E4B-8D96-0584CC53ABDB}"/>
+    <hyperlink ref="E39" r:id="rId176" xr:uid="{0C48DDBB-6D33-0647-BC8A-9CAF62245747}"/>
+    <hyperlink ref="D52" r:id="rId177" xr:uid="{C0863614-B91B-6045-9600-0C6554DFCC23}"/>
+    <hyperlink ref="E52" r:id="rId178" xr:uid="{6C53C8B6-B399-D54F-B2BD-ECFE9B0F0AEA}"/>
+    <hyperlink ref="D53" r:id="rId179" xr:uid="{D0DCE01E-C3C8-F042-9951-E28F6AAFBC52}"/>
+    <hyperlink ref="E53" r:id="rId180" xr:uid="{FEFFE228-358C-BB4B-811C-DF92C53065AF}"/>
+    <hyperlink ref="D105" r:id="rId181" xr:uid="{DBBFD5D1-31B9-614A-AF89-25FB0EAD3612}"/>
+    <hyperlink ref="E105" r:id="rId182" xr:uid="{9917BFA2-1C16-444A-9CF4-AEE99129AFE6}"/>
+    <hyperlink ref="D106" r:id="rId183" xr:uid="{59FD8485-695A-9C4F-A9D4-4428FBF03AE2}"/>
+    <hyperlink ref="E106" r:id="rId184" xr:uid="{BC4C20C3-1C6B-DE4E-8599-61CCD90A60ED}"/>
+    <hyperlink ref="D107" r:id="rId185" xr:uid="{3DDE3414-3549-4849-A386-0B6480CC15E5}"/>
+    <hyperlink ref="E107" r:id="rId186" xr:uid="{E9AF8289-8641-654D-9284-394FA6BB8074}"/>
+    <hyperlink ref="D108" r:id="rId187" xr:uid="{A4088AA3-8A95-954B-ABCD-FB6802B4AC4A}"/>
+    <hyperlink ref="E108" r:id="rId188" xr:uid="{624421EE-C5BA-D34B-8B6F-73F022187BC2}"/>
+    <hyperlink ref="D109" r:id="rId189" xr:uid="{40A0D934-1C7B-AD43-9FB3-8F9B20F3018B}"/>
+    <hyperlink ref="E109" r:id="rId190" xr:uid="{073CD9FD-81A7-9249-8EB3-544DFD00FFDD}"/>
+    <hyperlink ref="D124" r:id="rId191" xr:uid="{8AB277F3-D851-CC43-AE0D-F66E77CB9162}"/>
+    <hyperlink ref="E124" r:id="rId192" xr:uid="{98BF4EF1-B406-B748-8110-78C5C70143E3}"/>
+    <hyperlink ref="D125" r:id="rId193" xr:uid="{9FDDDDA0-167B-D141-9964-174A83CDD266}"/>
+    <hyperlink ref="E125" r:id="rId194" xr:uid="{7D633D57-A2CC-7D47-BF70-7886C95531B9}"/>
+    <hyperlink ref="D126" r:id="rId195" xr:uid="{06146951-1A1E-7D4A-9FF6-731ECC3946EE}"/>
+    <hyperlink ref="E126" r:id="rId196" xr:uid="{0851BE59-0EEE-534F-BA79-AE1A218495E3}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;"Aptos"&amp;10&amp;K000000 OFFICIAL&amp;1#_x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 OFFICIAL</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -6410,7 +10599,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C18CD9DC-A0FD-5B4E-8B82-402F8A51375A}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13"/>
@@ -6500,7 +10689,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>

</xml_diff>

<commit_message>
Final batch of manually scraped adopted plans
</commit_message>
<xml_diff>
--- a/data/manually_scraped_adopted_plans.xlsx
+++ b/data/manually_scraped_adopted_plans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sianteesdale/Documents/GitHub/local-plan-extractor/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28313B9-7C59-6044-B669-9EDF60B1801A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50851B5C-AE4F-2F4C-A0D4-9A099F7B1E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35800" windowHeight="26220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1937" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1937" uniqueCount="690">
   <si>
     <t>organisation</t>
   </si>
@@ -2102,6 +2102,9 @@
   </si>
   <si>
     <t>South Northamptonshire Council</t>
+  </si>
+  <si>
+    <t>https://somersetcc.sharepoint.com/:b:/s/SCCPublic/EXFQ-dSQ89JDh8h7E4tdfr0BnxcictPynUC3AphChUZoxw?e=CHWtPW</t>
   </si>
 </sst>
 </file>
@@ -2282,7 +2285,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2331,6 +2334,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5506,8 +5510,8 @@
       <c r="D105" s="41" t="s">
         <v>369</v>
       </c>
-      <c r="E105" s="41" t="s">
-        <v>370</v>
+      <c r="E105" s="48" t="s">
+        <v>689</v>
       </c>
       <c r="F105" s="16">
         <v>2006</v>
@@ -5532,7 +5536,7 @@
       <c r="C106" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="D106" s="41" t="s">
+      <c r="D106" s="48" t="s">
         <v>372</v>
       </c>
       <c r="E106" s="41" t="s">

</xml_diff>